<commit_message>
Consol TB report update 2026-03-14
</commit_message>
<xml_diff>
--- a/Consol_TB_FY25-26.xlsx
+++ b/Consol_TB_FY25-26.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8948" uniqueCount="362">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8933" uniqueCount="362">
   <si>
     <t>Book</t>
   </si>
@@ -1547,8 +1547,8 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{c005ace0-0bbc-41ee-a66e-108b9af6d1f8}">
-  <dimension ref="A1:I1788"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{26d2b73d-02bc-43c2-9043-7d317b793723}">
+  <dimension ref="A1:I1785"/>
   <sheetFormatPr defaultRowHeight="12.75"/>
   <cols>
     <col min="1" max="1" width="14.142857142857142" customWidth="1"/>
@@ -1787,10 +1787,10 @@
         <v>5.43186561E8</v>
       </c>
       <c r="H8" s="1">
-        <v>2.711028429799999E8</v>
+        <v>2.7110284297999996E8</v>
       </c>
       <c r="I8" s="1">
-        <v>2.720837180200001E8</v>
+        <v>2.7208371802000004E8</v>
       </c>
     </row>
     <row r="9" spans="1:9" ht="12.75">
@@ -3898,7 +3898,7 @@
         <v>13</v>
       </c>
       <c r="F81" s="1">
-        <v>0</v>
+        <v>-9.313225746154785E-10</v>
       </c>
       <c r="G81" s="1">
         <v>333614</v>
@@ -3907,7 +3907,7 @@
         <v>333614</v>
       </c>
       <c r="I81" s="1">
-        <v>0</v>
+        <v>-9.313225746154785E-10</v>
       </c>
     </row>
     <row r="82" spans="1:9" ht="12.75">
@@ -45252,7 +45252,7 @@
         <v>13</v>
       </c>
       <c r="F1507" s="1">
-        <v>-56797.000000002794</v>
+        <v>-56797.00000000186</v>
       </c>
       <c r="G1507" s="1">
         <v>3227421.9400000004</v>
@@ -45261,7 +45261,7 @@
         <v>3631156.939999997</v>
       </c>
       <c r="I1507" s="1">
-        <v>-460531.99999999953</v>
+        <v>-460531.9999999986</v>
       </c>
     </row>
     <row r="1508" spans="1:9" ht="12.75">
@@ -45310,7 +45310,7 @@
         <v>13</v>
       </c>
       <c r="F1509" s="1">
-        <v>0</v>
+        <v>-5.9604644775390625E-8</v>
       </c>
       <c r="G1509" s="1">
         <v>1.1068072367300003E9</v>
@@ -46302,10 +46302,10 @@
         <v>8.56587629E8</v>
       </c>
       <c r="H1543" s="1">
-        <v>3.3588584282E8</v>
+        <v>3.3588584282000005E8</v>
       </c>
       <c r="I1543" s="1">
-        <v>5.2070178618E8</v>
+        <v>5.2070178617999995E8</v>
       </c>
     </row>
     <row r="1544" spans="1:9" ht="12.75">
@@ -48265,19 +48265,19 @@
         <v>205</v>
       </c>
       <c r="E1611" t="s">
-        <v>13</v>
+        <v>329</v>
       </c>
       <c r="F1611" s="1">
         <v>0</v>
       </c>
       <c r="G1611" s="1">
-        <v>5901.95</v>
+        <v>1852706.82</v>
       </c>
       <c r="H1611" s="1">
         <v>0</v>
       </c>
       <c r="I1611" s="1">
-        <v>5901.95</v>
+        <v>1852706.82</v>
       </c>
     </row>
     <row r="1612" spans="1:9" ht="12.75">
@@ -48294,19 +48294,19 @@
         <v>205</v>
       </c>
       <c r="E1612" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="F1612" s="1">
         <v>0</v>
       </c>
       <c r="G1612" s="1">
-        <v>1852706.82</v>
+        <v>2174212.44</v>
       </c>
       <c r="H1612" s="1">
         <v>0</v>
       </c>
       <c r="I1612" s="1">
-        <v>1852706.82</v>
+        <v>2174212.44</v>
       </c>
     </row>
     <row r="1613" spans="1:9" ht="12.75">
@@ -48323,19 +48323,19 @@
         <v>205</v>
       </c>
       <c r="E1613" t="s">
-        <v>330</v>
+        <v>331</v>
       </c>
       <c r="F1613" s="1">
         <v>0</v>
       </c>
       <c r="G1613" s="1">
-        <v>2174212.44</v>
+        <v>2426050.95</v>
       </c>
       <c r="H1613" s="1">
         <v>0</v>
       </c>
       <c r="I1613" s="1">
-        <v>2174212.44</v>
+        <v>2426050.95</v>
       </c>
     </row>
     <row r="1614" spans="1:9" ht="12.75">
@@ -48352,19 +48352,19 @@
         <v>205</v>
       </c>
       <c r="E1614" t="s">
-        <v>331</v>
+        <v>333</v>
       </c>
       <c r="F1614" s="1">
         <v>0</v>
       </c>
       <c r="G1614" s="1">
-        <v>2420149</v>
+        <v>164829.20</v>
       </c>
       <c r="H1614" s="1">
         <v>0</v>
       </c>
       <c r="I1614" s="1">
-        <v>2420149</v>
+        <v>164829.20</v>
       </c>
     </row>
     <row r="1615" spans="1:9" ht="12.75">
@@ -48378,22 +48378,22 @@
         <v>105</v>
       </c>
       <c r="D1615" t="s">
-        <v>205</v>
+        <v>209</v>
       </c>
       <c r="E1615" t="s">
-        <v>333</v>
+        <v>331</v>
       </c>
       <c r="F1615" s="1">
         <v>0</v>
       </c>
       <c r="G1615" s="1">
-        <v>164829.20</v>
+        <v>1072113</v>
       </c>
       <c r="H1615" s="1">
         <v>0</v>
       </c>
       <c r="I1615" s="1">
-        <v>164829.20</v>
+        <v>1072113</v>
       </c>
     </row>
     <row r="1616" spans="1:9" ht="12.75">
@@ -48410,19 +48410,19 @@
         <v>209</v>
       </c>
       <c r="E1616" t="s">
-        <v>331</v>
+        <v>334</v>
       </c>
       <c r="F1616" s="1">
         <v>0</v>
       </c>
       <c r="G1616" s="1">
-        <v>1072113</v>
+        <v>145140</v>
       </c>
       <c r="H1616" s="1">
         <v>0</v>
       </c>
       <c r="I1616" s="1">
-        <v>1072113</v>
+        <v>145140</v>
       </c>
     </row>
     <row r="1617" spans="1:9" ht="12.75">
@@ -48439,7 +48439,7 @@
         <v>209</v>
       </c>
       <c r="E1617" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="F1617" s="1">
         <v>0</v>
@@ -48468,19 +48468,19 @@
         <v>209</v>
       </c>
       <c r="E1618" t="s">
-        <v>335</v>
+        <v>344</v>
       </c>
       <c r="F1618" s="1">
         <v>0</v>
       </c>
       <c r="G1618" s="1">
-        <v>145140</v>
+        <v>72570</v>
       </c>
       <c r="H1618" s="1">
         <v>0</v>
       </c>
       <c r="I1618" s="1">
-        <v>145140</v>
+        <v>72570</v>
       </c>
     </row>
     <row r="1619" spans="1:9" ht="12.75">
@@ -48497,7 +48497,7 @@
         <v>209</v>
       </c>
       <c r="E1619" t="s">
-        <v>344</v>
+        <v>337</v>
       </c>
       <c r="F1619" s="1">
         <v>0</v>
@@ -48526,19 +48526,19 @@
         <v>209</v>
       </c>
       <c r="E1620" t="s">
-        <v>337</v>
+        <v>345</v>
       </c>
       <c r="F1620" s="1">
         <v>0</v>
       </c>
       <c r="G1620" s="1">
-        <v>72570</v>
+        <v>842850</v>
       </c>
       <c r="H1620" s="1">
         <v>0</v>
       </c>
       <c r="I1620" s="1">
-        <v>72570</v>
+        <v>842850</v>
       </c>
     </row>
     <row r="1621" spans="1:9" ht="12.75">
@@ -48552,22 +48552,22 @@
         <v>105</v>
       </c>
       <c r="D1621" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="E1621" t="s">
-        <v>345</v>
+        <v>329</v>
       </c>
       <c r="F1621" s="1">
         <v>0</v>
       </c>
       <c r="G1621" s="1">
-        <v>842850</v>
+        <v>16809122</v>
       </c>
       <c r="H1621" s="1">
         <v>0</v>
       </c>
       <c r="I1621" s="1">
-        <v>842850</v>
+        <v>16809122</v>
       </c>
     </row>
     <row r="1622" spans="1:9" ht="12.75">
@@ -48584,19 +48584,19 @@
         <v>210</v>
       </c>
       <c r="E1622" t="s">
-        <v>13</v>
+        <v>330</v>
       </c>
       <c r="F1622" s="1">
         <v>0</v>
       </c>
       <c r="G1622" s="1">
-        <v>187655.03</v>
+        <v>11142323</v>
       </c>
       <c r="H1622" s="1">
         <v>0</v>
       </c>
       <c r="I1622" s="1">
-        <v>187655.03</v>
+        <v>11142323</v>
       </c>
     </row>
     <row r="1623" spans="1:9" ht="12.75">
@@ -48613,19 +48613,19 @@
         <v>210</v>
       </c>
       <c r="E1623" t="s">
-        <v>329</v>
+        <v>331</v>
       </c>
       <c r="F1623" s="1">
         <v>0</v>
       </c>
       <c r="G1623" s="1">
-        <v>16809122</v>
+        <v>7770928.95</v>
       </c>
       <c r="H1623" s="1">
         <v>0</v>
       </c>
       <c r="I1623" s="1">
-        <v>16809122</v>
+        <v>7770928.95</v>
       </c>
     </row>
     <row r="1624" spans="1:9" ht="12.75">
@@ -48642,19 +48642,19 @@
         <v>210</v>
       </c>
       <c r="E1624" t="s">
-        <v>330</v>
+        <v>332</v>
       </c>
       <c r="F1624" s="1">
         <v>0</v>
       </c>
       <c r="G1624" s="1">
-        <v>11142323</v>
+        <v>322143</v>
       </c>
       <c r="H1624" s="1">
         <v>0</v>
       </c>
       <c r="I1624" s="1">
-        <v>11142323</v>
+        <v>322143</v>
       </c>
     </row>
     <row r="1625" spans="1:9" ht="12.75">
@@ -48671,19 +48671,19 @@
         <v>210</v>
       </c>
       <c r="E1625" t="s">
-        <v>331</v>
+        <v>333</v>
       </c>
       <c r="F1625" s="1">
         <v>0</v>
       </c>
       <c r="G1625" s="1">
-        <v>7770928.95</v>
+        <v>152257</v>
       </c>
       <c r="H1625" s="1">
         <v>0</v>
       </c>
       <c r="I1625" s="1">
-        <v>7770928.95</v>
+        <v>152257</v>
       </c>
     </row>
     <row r="1626" spans="1:9" ht="12.75">
@@ -48700,19 +48700,19 @@
         <v>210</v>
       </c>
       <c r="E1626" t="s">
-        <v>332</v>
+        <v>334</v>
       </c>
       <c r="F1626" s="1">
         <v>0</v>
       </c>
       <c r="G1626" s="1">
-        <v>322143</v>
+        <v>1460685</v>
       </c>
       <c r="H1626" s="1">
         <v>0</v>
       </c>
       <c r="I1626" s="1">
-        <v>322143</v>
+        <v>1460685</v>
       </c>
     </row>
     <row r="1627" spans="1:9" ht="12.75">
@@ -48729,19 +48729,19 @@
         <v>210</v>
       </c>
       <c r="E1627" t="s">
-        <v>333</v>
+        <v>335</v>
       </c>
       <c r="F1627" s="1">
         <v>0</v>
       </c>
       <c r="G1627" s="1">
-        <v>152257</v>
+        <v>2802830</v>
       </c>
       <c r="H1627" s="1">
         <v>0</v>
       </c>
       <c r="I1627" s="1">
-        <v>152257</v>
+        <v>2802830</v>
       </c>
     </row>
     <row r="1628" spans="1:9" ht="12.75">
@@ -48758,19 +48758,19 @@
         <v>210</v>
       </c>
       <c r="E1628" t="s">
-        <v>334</v>
+        <v>336</v>
       </c>
       <c r="F1628" s="1">
         <v>0</v>
       </c>
       <c r="G1628" s="1">
-        <v>1460685</v>
+        <v>145830</v>
       </c>
       <c r="H1628" s="1">
         <v>0</v>
       </c>
       <c r="I1628" s="1">
-        <v>1460685</v>
+        <v>145830</v>
       </c>
     </row>
     <row r="1629" spans="1:9" ht="12.75">
@@ -48787,19 +48787,19 @@
         <v>210</v>
       </c>
       <c r="E1629" t="s">
-        <v>335</v>
+        <v>344</v>
       </c>
       <c r="F1629" s="1">
         <v>0</v>
       </c>
       <c r="G1629" s="1">
-        <v>2802830</v>
+        <v>271778</v>
       </c>
       <c r="H1629" s="1">
         <v>0</v>
       </c>
       <c r="I1629" s="1">
-        <v>2802830</v>
+        <v>271778</v>
       </c>
     </row>
     <row r="1630" spans="1:9" ht="12.75">
@@ -48816,19 +48816,19 @@
         <v>210</v>
       </c>
       <c r="E1630" t="s">
-        <v>336</v>
+        <v>337</v>
       </c>
       <c r="F1630" s="1">
         <v>0</v>
       </c>
       <c r="G1630" s="1">
-        <v>145830</v>
+        <v>442300</v>
       </c>
       <c r="H1630" s="1">
         <v>0</v>
       </c>
       <c r="I1630" s="1">
-        <v>145830</v>
+        <v>442300</v>
       </c>
     </row>
     <row r="1631" spans="1:9" ht="12.75">
@@ -48845,19 +48845,19 @@
         <v>210</v>
       </c>
       <c r="E1631" t="s">
-        <v>344</v>
+        <v>338</v>
       </c>
       <c r="F1631" s="1">
         <v>0</v>
       </c>
       <c r="G1631" s="1">
-        <v>271778</v>
+        <v>2881013</v>
       </c>
       <c r="H1631" s="1">
         <v>0</v>
       </c>
       <c r="I1631" s="1">
-        <v>271778</v>
+        <v>2881013</v>
       </c>
     </row>
     <row r="1632" spans="1:9" ht="12.75">
@@ -48874,19 +48874,19 @@
         <v>210</v>
       </c>
       <c r="E1632" t="s">
-        <v>337</v>
+        <v>339</v>
       </c>
       <c r="F1632" s="1">
         <v>0</v>
       </c>
       <c r="G1632" s="1">
-        <v>442300</v>
+        <v>47500</v>
       </c>
       <c r="H1632" s="1">
         <v>0</v>
       </c>
       <c r="I1632" s="1">
-        <v>442300</v>
+        <v>47500</v>
       </c>
     </row>
     <row r="1633" spans="1:9" ht="12.75">
@@ -48903,19 +48903,19 @@
         <v>210</v>
       </c>
       <c r="E1633" t="s">
-        <v>338</v>
+        <v>340</v>
       </c>
       <c r="F1633" s="1">
         <v>0</v>
       </c>
       <c r="G1633" s="1">
-        <v>2881013</v>
+        <v>61875</v>
       </c>
       <c r="H1633" s="1">
         <v>0</v>
       </c>
       <c r="I1633" s="1">
-        <v>2881013</v>
+        <v>61875</v>
       </c>
     </row>
     <row r="1634" spans="1:9" ht="12.75">
@@ -48932,19 +48932,19 @@
         <v>210</v>
       </c>
       <c r="E1634" t="s">
-        <v>339</v>
+        <v>341</v>
       </c>
       <c r="F1634" s="1">
         <v>0</v>
       </c>
       <c r="G1634" s="1">
-        <v>47500</v>
+        <v>1253200</v>
       </c>
       <c r="H1634" s="1">
         <v>0</v>
       </c>
       <c r="I1634" s="1">
-        <v>47500</v>
+        <v>1253200</v>
       </c>
     </row>
     <row r="1635" spans="1:9" ht="12.75">
@@ -48961,19 +48961,19 @@
         <v>210</v>
       </c>
       <c r="E1635" t="s">
-        <v>340</v>
+        <v>346</v>
       </c>
       <c r="F1635" s="1">
         <v>0</v>
       </c>
       <c r="G1635" s="1">
-        <v>61875</v>
+        <v>14465</v>
       </c>
       <c r="H1635" s="1">
         <v>0</v>
       </c>
       <c r="I1635" s="1">
-        <v>61875</v>
+        <v>14465</v>
       </c>
     </row>
     <row r="1636" spans="1:9" ht="12.75">
@@ -48990,19 +48990,19 @@
         <v>210</v>
       </c>
       <c r="E1636" t="s">
-        <v>341</v>
+        <v>347</v>
       </c>
       <c r="F1636" s="1">
         <v>0</v>
       </c>
       <c r="G1636" s="1">
-        <v>1173877.97</v>
+        <v>2458001</v>
       </c>
       <c r="H1636" s="1">
         <v>0</v>
       </c>
       <c r="I1636" s="1">
-        <v>1173877.97</v>
+        <v>2458001</v>
       </c>
     </row>
     <row r="1637" spans="1:9" ht="12.75">
@@ -49016,22 +49016,22 @@
         <v>105</v>
       </c>
       <c r="D1637" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="E1637" t="s">
-        <v>346</v>
+        <v>13</v>
       </c>
       <c r="F1637" s="1">
         <v>0</v>
       </c>
       <c r="G1637" s="1">
-        <v>14465</v>
+        <v>242538</v>
       </c>
       <c r="H1637" s="1">
         <v>0</v>
       </c>
       <c r="I1637" s="1">
-        <v>14465</v>
+        <v>242538</v>
       </c>
     </row>
     <row r="1638" spans="1:9" ht="12.75">
@@ -49045,22 +49045,22 @@
         <v>105</v>
       </c>
       <c r="D1638" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="E1638" t="s">
-        <v>347</v>
+        <v>329</v>
       </c>
       <c r="F1638" s="1">
         <v>0</v>
       </c>
       <c r="G1638" s="1">
-        <v>2349668</v>
+        <v>2133376.20</v>
       </c>
       <c r="H1638" s="1">
         <v>0</v>
       </c>
       <c r="I1638" s="1">
-        <v>2349668</v>
+        <v>2133376.20</v>
       </c>
     </row>
     <row r="1639" spans="1:9" ht="12.75">
@@ -49074,22 +49074,22 @@
         <v>105</v>
       </c>
       <c r="D1639" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="E1639" t="s">
-        <v>13</v>
+        <v>348</v>
       </c>
       <c r="F1639" s="1">
         <v>0</v>
       </c>
       <c r="G1639" s="1">
-        <v>242538</v>
+        <v>40134</v>
       </c>
       <c r="H1639" s="1">
         <v>0</v>
       </c>
       <c r="I1639" s="1">
-        <v>242538</v>
+        <v>40134</v>
       </c>
     </row>
     <row r="1640" spans="1:9" ht="12.75">
@@ -49106,19 +49106,19 @@
         <v>212</v>
       </c>
       <c r="E1640" t="s">
-        <v>13</v>
+        <v>330</v>
       </c>
       <c r="F1640" s="1">
         <v>0</v>
       </c>
       <c r="G1640" s="1">
-        <v>138819</v>
+        <v>2619977.68</v>
       </c>
       <c r="H1640" s="1">
         <v>0</v>
       </c>
       <c r="I1640" s="1">
-        <v>138819</v>
+        <v>2619977.68</v>
       </c>
     </row>
     <row r="1641" spans="1:9" ht="12.75">
@@ -49135,19 +49135,19 @@
         <v>212</v>
       </c>
       <c r="E1641" t="s">
-        <v>329</v>
+        <v>331</v>
       </c>
       <c r="F1641" s="1">
         <v>0</v>
       </c>
       <c r="G1641" s="1">
-        <v>2133376.20</v>
+        <v>2449797.92</v>
       </c>
       <c r="H1641" s="1">
         <v>0</v>
       </c>
       <c r="I1641" s="1">
-        <v>2133376.20</v>
+        <v>2449797.92</v>
       </c>
     </row>
     <row r="1642" spans="1:9" ht="12.75">
@@ -49164,19 +49164,19 @@
         <v>212</v>
       </c>
       <c r="E1642" t="s">
-        <v>348</v>
+        <v>332</v>
       </c>
       <c r="F1642" s="1">
         <v>0</v>
       </c>
       <c r="G1642" s="1">
-        <v>40134</v>
+        <v>578555</v>
       </c>
       <c r="H1642" s="1">
         <v>0</v>
       </c>
       <c r="I1642" s="1">
-        <v>40134</v>
+        <v>578555</v>
       </c>
     </row>
     <row r="1643" spans="1:9" ht="12.75">
@@ -49193,19 +49193,19 @@
         <v>212</v>
       </c>
       <c r="E1643" t="s">
-        <v>330</v>
+        <v>333</v>
       </c>
       <c r="F1643" s="1">
         <v>0</v>
       </c>
       <c r="G1643" s="1">
-        <v>2619977.6799999997</v>
+        <v>101989</v>
       </c>
       <c r="H1643" s="1">
         <v>0</v>
       </c>
       <c r="I1643" s="1">
-        <v>2619977.6799999997</v>
+        <v>101989</v>
       </c>
     </row>
     <row r="1644" spans="1:9" ht="12.75">
@@ -49222,19 +49222,19 @@
         <v>212</v>
       </c>
       <c r="E1644" t="s">
-        <v>331</v>
+        <v>349</v>
       </c>
       <c r="F1644" s="1">
         <v>0</v>
       </c>
       <c r="G1644" s="1">
-        <v>2404944.92</v>
+        <v>6559</v>
       </c>
       <c r="H1644" s="1">
         <v>0</v>
       </c>
       <c r="I1644" s="1">
-        <v>2404944.92</v>
+        <v>6559</v>
       </c>
     </row>
     <row r="1645" spans="1:9" ht="12.75">
@@ -49251,19 +49251,19 @@
         <v>212</v>
       </c>
       <c r="E1645" t="s">
-        <v>332</v>
+        <v>334</v>
       </c>
       <c r="F1645" s="1">
         <v>0</v>
       </c>
       <c r="G1645" s="1">
-        <v>578555</v>
+        <v>200632</v>
       </c>
       <c r="H1645" s="1">
         <v>0</v>
       </c>
       <c r="I1645" s="1">
-        <v>578555</v>
+        <v>200632</v>
       </c>
     </row>
     <row r="1646" spans="1:9" ht="12.75">
@@ -49280,19 +49280,19 @@
         <v>212</v>
       </c>
       <c r="E1646" t="s">
-        <v>333</v>
+        <v>350</v>
       </c>
       <c r="F1646" s="1">
         <v>0</v>
       </c>
       <c r="G1646" s="1">
-        <v>101989</v>
+        <v>13921</v>
       </c>
       <c r="H1646" s="1">
         <v>0</v>
       </c>
       <c r="I1646" s="1">
-        <v>101989</v>
+        <v>13921</v>
       </c>
     </row>
     <row r="1647" spans="1:9" ht="12.75">
@@ -49309,19 +49309,19 @@
         <v>212</v>
       </c>
       <c r="E1647" t="s">
-        <v>349</v>
+        <v>335</v>
       </c>
       <c r="F1647" s="1">
         <v>0</v>
       </c>
       <c r="G1647" s="1">
-        <v>6559</v>
+        <v>3436</v>
       </c>
       <c r="H1647" s="1">
         <v>0</v>
       </c>
       <c r="I1647" s="1">
-        <v>6559</v>
+        <v>3436</v>
       </c>
     </row>
     <row r="1648" spans="1:9" ht="12.75">
@@ -49338,19 +49338,19 @@
         <v>212</v>
       </c>
       <c r="E1648" t="s">
-        <v>334</v>
+        <v>338</v>
       </c>
       <c r="F1648" s="1">
         <v>0</v>
       </c>
       <c r="G1648" s="1">
-        <v>200632</v>
+        <v>300656</v>
       </c>
       <c r="H1648" s="1">
         <v>0</v>
       </c>
       <c r="I1648" s="1">
-        <v>200632</v>
+        <v>300656</v>
       </c>
     </row>
     <row r="1649" spans="1:9" ht="12.75">
@@ -49367,19 +49367,19 @@
         <v>212</v>
       </c>
       <c r="E1649" t="s">
-        <v>350</v>
+        <v>346</v>
       </c>
       <c r="F1649" s="1">
         <v>0</v>
       </c>
       <c r="G1649" s="1">
-        <v>13921</v>
+        <v>1144422</v>
       </c>
       <c r="H1649" s="1">
         <v>0</v>
       </c>
       <c r="I1649" s="1">
-        <v>13921</v>
+        <v>1144422</v>
       </c>
     </row>
     <row r="1650" spans="1:9" ht="12.75">
@@ -49393,22 +49393,22 @@
         <v>105</v>
       </c>
       <c r="D1650" t="s">
-        <v>212</v>
+        <v>218</v>
       </c>
       <c r="E1650" t="s">
-        <v>335</v>
+        <v>343</v>
       </c>
       <c r="F1650" s="1">
         <v>0</v>
       </c>
       <c r="G1650" s="1">
-        <v>3436</v>
+        <v>1824</v>
       </c>
       <c r="H1650" s="1">
         <v>0</v>
       </c>
       <c r="I1650" s="1">
-        <v>3436</v>
+        <v>1824</v>
       </c>
     </row>
     <row r="1651" spans="1:9" ht="12.75">
@@ -49422,22 +49422,22 @@
         <v>105</v>
       </c>
       <c r="D1651" t="s">
-        <v>212</v>
+        <v>218</v>
       </c>
       <c r="E1651" t="s">
-        <v>338</v>
+        <v>339</v>
       </c>
       <c r="F1651" s="1">
         <v>0</v>
       </c>
       <c r="G1651" s="1">
-        <v>286496</v>
+        <v>223551</v>
       </c>
       <c r="H1651" s="1">
         <v>0</v>
       </c>
       <c r="I1651" s="1">
-        <v>286496</v>
+        <v>223551</v>
       </c>
     </row>
     <row r="1652" spans="1:9" ht="12.75">
@@ -49451,22 +49451,22 @@
         <v>105</v>
       </c>
       <c r="D1652" t="s">
-        <v>212</v>
+        <v>219</v>
       </c>
       <c r="E1652" t="s">
-        <v>346</v>
+        <v>329</v>
       </c>
       <c r="F1652" s="1">
         <v>0</v>
       </c>
       <c r="G1652" s="1">
-        <v>1064616</v>
+        <v>49500</v>
       </c>
       <c r="H1652" s="1">
         <v>0</v>
       </c>
       <c r="I1652" s="1">
-        <v>1064616</v>
+        <v>49500</v>
       </c>
     </row>
     <row r="1653" spans="1:9" ht="12.75">
@@ -49480,22 +49480,22 @@
         <v>105</v>
       </c>
       <c r="D1653" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="E1653" t="s">
-        <v>343</v>
+        <v>331</v>
       </c>
       <c r="F1653" s="1">
         <v>0</v>
       </c>
       <c r="G1653" s="1">
-        <v>1824</v>
+        <v>2507503</v>
       </c>
       <c r="H1653" s="1">
         <v>0</v>
       </c>
       <c r="I1653" s="1">
-        <v>1824</v>
+        <v>2507503</v>
       </c>
     </row>
     <row r="1654" spans="1:9" ht="12.75">
@@ -49509,22 +49509,22 @@
         <v>105</v>
       </c>
       <c r="D1654" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="E1654" t="s">
-        <v>339</v>
+        <v>332</v>
       </c>
       <c r="F1654" s="1">
         <v>0</v>
       </c>
       <c r="G1654" s="1">
-        <v>223551</v>
+        <v>65932</v>
       </c>
       <c r="H1654" s="1">
         <v>0</v>
       </c>
       <c r="I1654" s="1">
-        <v>223551</v>
+        <v>65932</v>
       </c>
     </row>
     <row r="1655" spans="1:9" ht="12.75">
@@ -49541,19 +49541,19 @@
         <v>219</v>
       </c>
       <c r="E1655" t="s">
-        <v>329</v>
+        <v>333</v>
       </c>
       <c r="F1655" s="1">
         <v>0</v>
       </c>
       <c r="G1655" s="1">
-        <v>49500</v>
+        <v>86124</v>
       </c>
       <c r="H1655" s="1">
         <v>0</v>
       </c>
       <c r="I1655" s="1">
-        <v>49500</v>
+        <v>86124</v>
       </c>
     </row>
     <row r="1656" spans="1:9" ht="12.75">
@@ -49570,19 +49570,19 @@
         <v>219</v>
       </c>
       <c r="E1656" t="s">
-        <v>331</v>
+        <v>334</v>
       </c>
       <c r="F1656" s="1">
         <v>0</v>
       </c>
       <c r="G1656" s="1">
-        <v>2507503</v>
+        <v>1021380</v>
       </c>
       <c r="H1656" s="1">
         <v>0</v>
       </c>
       <c r="I1656" s="1">
-        <v>2507503</v>
+        <v>1021380</v>
       </c>
     </row>
     <row r="1657" spans="1:9" ht="12.75">
@@ -49599,19 +49599,19 @@
         <v>219</v>
       </c>
       <c r="E1657" t="s">
-        <v>332</v>
+        <v>335</v>
       </c>
       <c r="F1657" s="1">
         <v>0</v>
       </c>
       <c r="G1657" s="1">
-        <v>65932</v>
+        <v>138789</v>
       </c>
       <c r="H1657" s="1">
         <v>0</v>
       </c>
       <c r="I1657" s="1">
-        <v>65932</v>
+        <v>138789</v>
       </c>
     </row>
     <row r="1658" spans="1:9" ht="12.75">
@@ -49628,19 +49628,19 @@
         <v>219</v>
       </c>
       <c r="E1658" t="s">
-        <v>333</v>
+        <v>336</v>
       </c>
       <c r="F1658" s="1">
         <v>0</v>
       </c>
       <c r="G1658" s="1">
-        <v>86124</v>
+        <v>8288</v>
       </c>
       <c r="H1658" s="1">
         <v>0</v>
       </c>
       <c r="I1658" s="1">
-        <v>86124</v>
+        <v>8288</v>
       </c>
     </row>
     <row r="1659" spans="1:9" ht="12.75">
@@ -49657,19 +49657,19 @@
         <v>219</v>
       </c>
       <c r="E1659" t="s">
-        <v>334</v>
+        <v>338</v>
       </c>
       <c r="F1659" s="1">
         <v>0</v>
       </c>
       <c r="G1659" s="1">
-        <v>1021380</v>
+        <v>219258</v>
       </c>
       <c r="H1659" s="1">
         <v>0</v>
       </c>
       <c r="I1659" s="1">
-        <v>1021380</v>
+        <v>219258</v>
       </c>
     </row>
     <row r="1660" spans="1:9" ht="12.75">
@@ -49686,19 +49686,19 @@
         <v>219</v>
       </c>
       <c r="E1660" t="s">
-        <v>335</v>
+        <v>339</v>
       </c>
       <c r="F1660" s="1">
         <v>0</v>
       </c>
       <c r="G1660" s="1">
-        <v>138789</v>
+        <v>4807583</v>
       </c>
       <c r="H1660" s="1">
-        <v>0</v>
+        <v>4807583</v>
       </c>
       <c r="I1660" s="1">
-        <v>138789</v>
+        <v>0</v>
       </c>
     </row>
     <row r="1661" spans="1:9" ht="12.75">
@@ -49715,19 +49715,19 @@
         <v>219</v>
       </c>
       <c r="E1661" t="s">
-        <v>336</v>
+        <v>341</v>
       </c>
       <c r="F1661" s="1">
         <v>0</v>
       </c>
       <c r="G1661" s="1">
-        <v>8288</v>
+        <v>13811</v>
       </c>
       <c r="H1661" s="1">
         <v>0</v>
       </c>
       <c r="I1661" s="1">
-        <v>8288</v>
+        <v>13811</v>
       </c>
     </row>
     <row r="1662" spans="1:9" ht="12.75">
@@ -49744,19 +49744,19 @@
         <v>219</v>
       </c>
       <c r="E1662" t="s">
-        <v>338</v>
+        <v>342</v>
       </c>
       <c r="F1662" s="1">
         <v>0</v>
       </c>
       <c r="G1662" s="1">
-        <v>219258</v>
+        <v>729998</v>
       </c>
       <c r="H1662" s="1">
         <v>0</v>
       </c>
       <c r="I1662" s="1">
-        <v>219258</v>
+        <v>729998</v>
       </c>
     </row>
     <row r="1663" spans="1:9" ht="12.75">
@@ -49770,22 +49770,22 @@
         <v>105</v>
       </c>
       <c r="D1663" t="s">
-        <v>219</v>
+        <v>221</v>
       </c>
       <c r="E1663" t="s">
-        <v>339</v>
+        <v>331</v>
       </c>
       <c r="F1663" s="1">
         <v>0</v>
       </c>
       <c r="G1663" s="1">
-        <v>4807583</v>
+        <v>3734639.2300000004</v>
       </c>
       <c r="H1663" s="1">
-        <v>4807583</v>
+        <v>0</v>
       </c>
       <c r="I1663" s="1">
-        <v>0</v>
+        <v>3734639.2300000004</v>
       </c>
     </row>
     <row r="1664" spans="1:9" ht="12.75">
@@ -49799,22 +49799,22 @@
         <v>105</v>
       </c>
       <c r="D1664" t="s">
-        <v>219</v>
+        <v>221</v>
       </c>
       <c r="E1664" t="s">
-        <v>341</v>
+        <v>332</v>
       </c>
       <c r="F1664" s="1">
         <v>0</v>
       </c>
       <c r="G1664" s="1">
-        <v>13811</v>
+        <v>289295.48</v>
       </c>
       <c r="H1664" s="1">
         <v>0</v>
       </c>
       <c r="I1664" s="1">
-        <v>13811</v>
+        <v>289295.48</v>
       </c>
     </row>
     <row r="1665" spans="1:9" ht="12.75">
@@ -49828,22 +49828,22 @@
         <v>105</v>
       </c>
       <c r="D1665" t="s">
-        <v>219</v>
+        <v>221</v>
       </c>
       <c r="E1665" t="s">
-        <v>342</v>
+        <v>333</v>
       </c>
       <c r="F1665" s="1">
         <v>0</v>
       </c>
       <c r="G1665" s="1">
-        <v>729998</v>
+        <v>218609.22</v>
       </c>
       <c r="H1665" s="1">
         <v>0</v>
       </c>
       <c r="I1665" s="1">
-        <v>729998</v>
+        <v>218609.22</v>
       </c>
     </row>
     <row r="1666" spans="1:9" ht="12.75">
@@ -49860,19 +49860,19 @@
         <v>221</v>
       </c>
       <c r="E1666" t="s">
-        <v>331</v>
+        <v>334</v>
       </c>
       <c r="F1666" s="1">
         <v>0</v>
       </c>
       <c r="G1666" s="1">
-        <v>3734639.2300000004</v>
+        <v>1910663.08</v>
       </c>
       <c r="H1666" s="1">
         <v>0</v>
       </c>
       <c r="I1666" s="1">
-        <v>3734639.2300000004</v>
+        <v>1910663.08</v>
       </c>
     </row>
     <row r="1667" spans="1:9" ht="12.75">
@@ -49889,19 +49889,19 @@
         <v>221</v>
       </c>
       <c r="E1667" t="s">
-        <v>332</v>
+        <v>335</v>
       </c>
       <c r="F1667" s="1">
         <v>0</v>
       </c>
       <c r="G1667" s="1">
-        <v>289295.48</v>
+        <v>685737.6099999999</v>
       </c>
       <c r="H1667" s="1">
         <v>0</v>
       </c>
       <c r="I1667" s="1">
-        <v>289295.48</v>
+        <v>685737.6099999999</v>
       </c>
     </row>
     <row r="1668" spans="1:9" ht="12.75">
@@ -49918,19 +49918,19 @@
         <v>221</v>
       </c>
       <c r="E1668" t="s">
-        <v>333</v>
+        <v>336</v>
       </c>
       <c r="F1668" s="1">
         <v>0</v>
       </c>
       <c r="G1668" s="1">
-        <v>218609.22</v>
+        <v>4078.70</v>
       </c>
       <c r="H1668" s="1">
         <v>0</v>
       </c>
       <c r="I1668" s="1">
-        <v>218609.22</v>
+        <v>4078.70</v>
       </c>
     </row>
     <row r="1669" spans="1:9" ht="12.75">
@@ -49947,19 +49947,19 @@
         <v>221</v>
       </c>
       <c r="E1669" t="s">
-        <v>334</v>
+        <v>337</v>
       </c>
       <c r="F1669" s="1">
         <v>0</v>
       </c>
       <c r="G1669" s="1">
-        <v>1910663.0799999998</v>
+        <v>191355.02000000002</v>
       </c>
       <c r="H1669" s="1">
         <v>0</v>
       </c>
       <c r="I1669" s="1">
-        <v>1910663.0799999998</v>
+        <v>191355.02000000002</v>
       </c>
     </row>
     <row r="1670" spans="1:9" ht="12.75">
@@ -49976,19 +49976,19 @@
         <v>221</v>
       </c>
       <c r="E1670" t="s">
-        <v>335</v>
+        <v>338</v>
       </c>
       <c r="F1670" s="1">
         <v>0</v>
       </c>
       <c r="G1670" s="1">
-        <v>685737.61</v>
+        <v>381348.32000000007</v>
       </c>
       <c r="H1670" s="1">
         <v>0</v>
       </c>
       <c r="I1670" s="1">
-        <v>685737.61</v>
+        <v>381348.32000000007</v>
       </c>
     </row>
     <row r="1671" spans="1:9" ht="12.75">
@@ -50005,19 +50005,19 @@
         <v>221</v>
       </c>
       <c r="E1671" t="s">
-        <v>336</v>
+        <v>340</v>
       </c>
       <c r="F1671" s="1">
         <v>0</v>
       </c>
       <c r="G1671" s="1">
-        <v>4078.70</v>
+        <v>93497</v>
       </c>
       <c r="H1671" s="1">
         <v>0</v>
       </c>
       <c r="I1671" s="1">
-        <v>4078.70</v>
+        <v>93497</v>
       </c>
     </row>
     <row r="1672" spans="1:9" ht="12.75">
@@ -50034,19 +50034,19 @@
         <v>221</v>
       </c>
       <c r="E1672" t="s">
-        <v>337</v>
+        <v>341</v>
       </c>
       <c r="F1672" s="1">
         <v>0</v>
       </c>
       <c r="G1672" s="1">
-        <v>191355.02000000002</v>
+        <v>211054</v>
       </c>
       <c r="H1672" s="1">
         <v>0</v>
       </c>
       <c r="I1672" s="1">
-        <v>191355.02000000002</v>
+        <v>211054</v>
       </c>
     </row>
     <row r="1673" spans="1:9" ht="12.75">
@@ -50063,19 +50063,19 @@
         <v>221</v>
       </c>
       <c r="E1673" t="s">
-        <v>338</v>
+        <v>342</v>
       </c>
       <c r="F1673" s="1">
         <v>0</v>
       </c>
       <c r="G1673" s="1">
-        <v>381348.32</v>
+        <v>1105942</v>
       </c>
       <c r="H1673" s="1">
         <v>0</v>
       </c>
       <c r="I1673" s="1">
-        <v>381348.32</v>
+        <v>1105942</v>
       </c>
     </row>
     <row r="1674" spans="1:9" ht="12.75">
@@ -50089,22 +50089,22 @@
         <v>105</v>
       </c>
       <c r="D1674" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="E1674" t="s">
-        <v>340</v>
+        <v>329</v>
       </c>
       <c r="F1674" s="1">
         <v>0</v>
       </c>
       <c r="G1674" s="1">
-        <v>93497</v>
+        <v>1711047.58</v>
       </c>
       <c r="H1674" s="1">
         <v>0</v>
       </c>
       <c r="I1674" s="1">
-        <v>93497</v>
+        <v>1711047.58</v>
       </c>
     </row>
     <row r="1675" spans="1:9" ht="12.75">
@@ -50118,22 +50118,22 @@
         <v>105</v>
       </c>
       <c r="D1675" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="E1675" t="s">
-        <v>341</v>
+        <v>330</v>
       </c>
       <c r="F1675" s="1">
         <v>0</v>
       </c>
       <c r="G1675" s="1">
-        <v>211054</v>
+        <v>1338867.5899999999</v>
       </c>
       <c r="H1675" s="1">
         <v>0</v>
       </c>
       <c r="I1675" s="1">
-        <v>211054</v>
+        <v>1338867.5899999999</v>
       </c>
     </row>
     <row r="1676" spans="1:9" ht="12.75">
@@ -50147,22 +50147,22 @@
         <v>105</v>
       </c>
       <c r="D1676" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="E1676" t="s">
-        <v>342</v>
+        <v>331</v>
       </c>
       <c r="F1676" s="1">
         <v>0</v>
       </c>
       <c r="G1676" s="1">
-        <v>1105942</v>
+        <v>6084145</v>
       </c>
       <c r="H1676" s="1">
         <v>0</v>
       </c>
       <c r="I1676" s="1">
-        <v>1105942</v>
+        <v>6084145</v>
       </c>
     </row>
     <row r="1677" spans="1:9" ht="12.75">
@@ -50179,19 +50179,19 @@
         <v>222</v>
       </c>
       <c r="E1677" t="s">
-        <v>329</v>
+        <v>332</v>
       </c>
       <c r="F1677" s="1">
         <v>0</v>
       </c>
       <c r="G1677" s="1">
-        <v>1711047.58</v>
+        <v>492996</v>
       </c>
       <c r="H1677" s="1">
         <v>0</v>
       </c>
       <c r="I1677" s="1">
-        <v>1711047.58</v>
+        <v>492996</v>
       </c>
     </row>
     <row r="1678" spans="1:9" ht="12.75">
@@ -50208,19 +50208,19 @@
         <v>222</v>
       </c>
       <c r="E1678" t="s">
-        <v>330</v>
+        <v>333</v>
       </c>
       <c r="F1678" s="1">
         <v>0</v>
       </c>
       <c r="G1678" s="1">
-        <v>1338867.5899999999</v>
+        <v>351533</v>
       </c>
       <c r="H1678" s="1">
         <v>0</v>
       </c>
       <c r="I1678" s="1">
-        <v>1338867.5899999999</v>
+        <v>351533</v>
       </c>
     </row>
     <row r="1679" spans="1:9" ht="12.75">
@@ -50237,19 +50237,19 @@
         <v>222</v>
       </c>
       <c r="E1679" t="s">
-        <v>331</v>
+        <v>334</v>
       </c>
       <c r="F1679" s="1">
         <v>0</v>
       </c>
       <c r="G1679" s="1">
-        <v>6084145</v>
+        <v>10682502</v>
       </c>
       <c r="H1679" s="1">
         <v>0</v>
       </c>
       <c r="I1679" s="1">
-        <v>6084145</v>
+        <v>10682502</v>
       </c>
     </row>
     <row r="1680" spans="1:9" ht="12.75">
@@ -50266,19 +50266,19 @@
         <v>222</v>
       </c>
       <c r="E1680" t="s">
-        <v>332</v>
+        <v>335</v>
       </c>
       <c r="F1680" s="1">
         <v>0</v>
       </c>
       <c r="G1680" s="1">
-        <v>492996</v>
+        <v>992656</v>
       </c>
       <c r="H1680" s="1">
         <v>0</v>
       </c>
       <c r="I1680" s="1">
-        <v>492996</v>
+        <v>992656</v>
       </c>
     </row>
     <row r="1681" spans="1:9" ht="12.75">
@@ -50295,19 +50295,19 @@
         <v>222</v>
       </c>
       <c r="E1681" t="s">
-        <v>333</v>
+        <v>336</v>
       </c>
       <c r="F1681" s="1">
         <v>0</v>
       </c>
       <c r="G1681" s="1">
-        <v>351533</v>
+        <v>12048</v>
       </c>
       <c r="H1681" s="1">
         <v>0</v>
       </c>
       <c r="I1681" s="1">
-        <v>351533</v>
+        <v>12048</v>
       </c>
     </row>
     <row r="1682" spans="1:9" ht="12.75">
@@ -50324,19 +50324,19 @@
         <v>222</v>
       </c>
       <c r="E1682" t="s">
-        <v>334</v>
+        <v>344</v>
       </c>
       <c r="F1682" s="1">
         <v>0</v>
       </c>
       <c r="G1682" s="1">
-        <v>10682502</v>
+        <v>25244</v>
       </c>
       <c r="H1682" s="1">
         <v>0</v>
       </c>
       <c r="I1682" s="1">
-        <v>10682502</v>
+        <v>25244</v>
       </c>
     </row>
     <row r="1683" spans="1:9" ht="12.75">
@@ -50353,19 +50353,19 @@
         <v>222</v>
       </c>
       <c r="E1683" t="s">
-        <v>335</v>
+        <v>337</v>
       </c>
       <c r="F1683" s="1">
         <v>0</v>
       </c>
       <c r="G1683" s="1">
-        <v>992656</v>
+        <v>288601</v>
       </c>
       <c r="H1683" s="1">
         <v>0</v>
       </c>
       <c r="I1683" s="1">
-        <v>992656</v>
+        <v>288601</v>
       </c>
     </row>
     <row r="1684" spans="1:9" ht="12.75">
@@ -50382,19 +50382,19 @@
         <v>222</v>
       </c>
       <c r="E1684" t="s">
-        <v>336</v>
+        <v>338</v>
       </c>
       <c r="F1684" s="1">
         <v>0</v>
       </c>
       <c r="G1684" s="1">
-        <v>12048</v>
+        <v>1595017</v>
       </c>
       <c r="H1684" s="1">
         <v>0</v>
       </c>
       <c r="I1684" s="1">
-        <v>12048</v>
+        <v>1595017</v>
       </c>
     </row>
     <row r="1685" spans="1:9" ht="12.75">
@@ -50411,19 +50411,19 @@
         <v>222</v>
       </c>
       <c r="E1685" t="s">
-        <v>344</v>
+        <v>351</v>
       </c>
       <c r="F1685" s="1">
         <v>0</v>
       </c>
       <c r="G1685" s="1">
-        <v>25244</v>
+        <v>100146</v>
       </c>
       <c r="H1685" s="1">
         <v>0</v>
       </c>
       <c r="I1685" s="1">
-        <v>25244</v>
+        <v>100146</v>
       </c>
     </row>
     <row r="1686" spans="1:9" ht="12.75">
@@ -50440,19 +50440,19 @@
         <v>222</v>
       </c>
       <c r="E1686" t="s">
-        <v>337</v>
+        <v>352</v>
       </c>
       <c r="F1686" s="1">
         <v>0</v>
       </c>
       <c r="G1686" s="1">
-        <v>288601</v>
+        <v>279211</v>
       </c>
       <c r="H1686" s="1">
         <v>0</v>
       </c>
       <c r="I1686" s="1">
-        <v>288601</v>
+        <v>279211</v>
       </c>
     </row>
     <row r="1687" spans="1:9" ht="12.75">
@@ -50469,19 +50469,19 @@
         <v>222</v>
       </c>
       <c r="E1687" t="s">
-        <v>338</v>
+        <v>353</v>
       </c>
       <c r="F1687" s="1">
         <v>0</v>
       </c>
       <c r="G1687" s="1">
-        <v>1595017</v>
+        <v>227931</v>
       </c>
       <c r="H1687" s="1">
         <v>0</v>
       </c>
       <c r="I1687" s="1">
-        <v>1595017</v>
+        <v>227931</v>
       </c>
     </row>
     <row r="1688" spans="1:9" ht="12.75">
@@ -50498,19 +50498,19 @@
         <v>222</v>
       </c>
       <c r="E1688" t="s">
-        <v>351</v>
+        <v>354</v>
       </c>
       <c r="F1688" s="1">
         <v>0</v>
       </c>
       <c r="G1688" s="1">
-        <v>100146</v>
+        <v>53925</v>
       </c>
       <c r="H1688" s="1">
         <v>0</v>
       </c>
       <c r="I1688" s="1">
-        <v>100146</v>
+        <v>53925</v>
       </c>
     </row>
     <row r="1689" spans="1:9" ht="12.75">
@@ -50524,22 +50524,22 @@
         <v>105</v>
       </c>
       <c r="D1689" t="s">
-        <v>222</v>
+        <v>224</v>
       </c>
       <c r="E1689" t="s">
-        <v>352</v>
+        <v>348</v>
       </c>
       <c r="F1689" s="1">
         <v>0</v>
       </c>
       <c r="G1689" s="1">
-        <v>279211</v>
+        <v>0</v>
       </c>
       <c r="H1689" s="1">
-        <v>0</v>
+        <v>2.423587017E7</v>
       </c>
       <c r="I1689" s="1">
-        <v>279211</v>
+        <v>-2.423587017E7</v>
       </c>
     </row>
     <row r="1690" spans="1:9" ht="12.75">
@@ -50553,22 +50553,22 @@
         <v>105</v>
       </c>
       <c r="D1690" t="s">
-        <v>222</v>
+        <v>225</v>
       </c>
       <c r="E1690" t="s">
-        <v>353</v>
+        <v>348</v>
       </c>
       <c r="F1690" s="1">
         <v>0</v>
       </c>
       <c r="G1690" s="1">
-        <v>227931</v>
+        <v>119165</v>
       </c>
       <c r="H1690" s="1">
         <v>0</v>
       </c>
       <c r="I1690" s="1">
-        <v>227931</v>
+        <v>119165</v>
       </c>
     </row>
     <row r="1691" spans="1:9" ht="12.75">
@@ -50582,22 +50582,22 @@
         <v>105</v>
       </c>
       <c r="D1691" t="s">
-        <v>222</v>
+        <v>307</v>
       </c>
       <c r="E1691" t="s">
-        <v>354</v>
+        <v>329</v>
       </c>
       <c r="F1691" s="1">
         <v>0</v>
       </c>
       <c r="G1691" s="1">
-        <v>53925</v>
+        <v>10532</v>
       </c>
       <c r="H1691" s="1">
         <v>0</v>
       </c>
       <c r="I1691" s="1">
-        <v>53925</v>
+        <v>10532</v>
       </c>
     </row>
     <row r="1692" spans="1:9" ht="12.75">
@@ -50611,22 +50611,22 @@
         <v>105</v>
       </c>
       <c r="D1692" t="s">
-        <v>224</v>
+        <v>307</v>
       </c>
       <c r="E1692" t="s">
-        <v>348</v>
+        <v>330</v>
       </c>
       <c r="F1692" s="1">
         <v>0</v>
       </c>
       <c r="G1692" s="1">
-        <v>0</v>
+        <v>1417</v>
       </c>
       <c r="H1692" s="1">
-        <v>2.423587017E7</v>
+        <v>0</v>
       </c>
       <c r="I1692" s="1">
-        <v>-2.423587017E7</v>
+        <v>1417</v>
       </c>
     </row>
     <row r="1693" spans="1:9" ht="12.75">
@@ -50640,22 +50640,22 @@
         <v>105</v>
       </c>
       <c r="D1693" t="s">
-        <v>225</v>
+        <v>307</v>
       </c>
       <c r="E1693" t="s">
-        <v>348</v>
+        <v>331</v>
       </c>
       <c r="F1693" s="1">
         <v>0</v>
       </c>
       <c r="G1693" s="1">
-        <v>119165</v>
+        <v>88200</v>
       </c>
       <c r="H1693" s="1">
         <v>0</v>
       </c>
       <c r="I1693" s="1">
-        <v>119165</v>
+        <v>88200</v>
       </c>
     </row>
     <row r="1694" spans="1:9" ht="12.75">
@@ -50672,19 +50672,19 @@
         <v>307</v>
       </c>
       <c r="E1694" t="s">
-        <v>329</v>
+        <v>332</v>
       </c>
       <c r="F1694" s="1">
         <v>0</v>
       </c>
       <c r="G1694" s="1">
-        <v>10532</v>
+        <v>3374</v>
       </c>
       <c r="H1694" s="1">
         <v>0</v>
       </c>
       <c r="I1694" s="1">
-        <v>10532</v>
+        <v>3374</v>
       </c>
     </row>
     <row r="1695" spans="1:9" ht="12.75">
@@ -50701,19 +50701,19 @@
         <v>307</v>
       </c>
       <c r="E1695" t="s">
-        <v>330</v>
+        <v>333</v>
       </c>
       <c r="F1695" s="1">
         <v>0</v>
       </c>
       <c r="G1695" s="1">
-        <v>1417</v>
+        <v>5996</v>
       </c>
       <c r="H1695" s="1">
         <v>0</v>
       </c>
       <c r="I1695" s="1">
-        <v>1417</v>
+        <v>5996</v>
       </c>
     </row>
     <row r="1696" spans="1:9" ht="12.75">
@@ -50730,19 +50730,19 @@
         <v>307</v>
       </c>
       <c r="E1696" t="s">
-        <v>331</v>
+        <v>334</v>
       </c>
       <c r="F1696" s="1">
         <v>0</v>
       </c>
       <c r="G1696" s="1">
-        <v>88200</v>
+        <v>22800</v>
       </c>
       <c r="H1696" s="1">
         <v>0</v>
       </c>
       <c r="I1696" s="1">
-        <v>88200</v>
+        <v>22800</v>
       </c>
     </row>
     <row r="1697" spans="1:9" ht="12.75">
@@ -50759,19 +50759,19 @@
         <v>307</v>
       </c>
       <c r="E1697" t="s">
-        <v>332</v>
+        <v>335</v>
       </c>
       <c r="F1697" s="1">
         <v>0</v>
       </c>
       <c r="G1697" s="1">
-        <v>3374</v>
+        <v>12631</v>
       </c>
       <c r="H1697" s="1">
         <v>0</v>
       </c>
       <c r="I1697" s="1">
-        <v>3374</v>
+        <v>12631</v>
       </c>
     </row>
     <row r="1698" spans="1:9" ht="12.75">
@@ -50788,19 +50788,19 @@
         <v>307</v>
       </c>
       <c r="E1698" t="s">
-        <v>333</v>
+        <v>336</v>
       </c>
       <c r="F1698" s="1">
         <v>0</v>
       </c>
       <c r="G1698" s="1">
-        <v>5996</v>
+        <v>179</v>
       </c>
       <c r="H1698" s="1">
         <v>0</v>
       </c>
       <c r="I1698" s="1">
-        <v>5996</v>
+        <v>179</v>
       </c>
     </row>
     <row r="1699" spans="1:9" ht="12.75">
@@ -50817,19 +50817,19 @@
         <v>307</v>
       </c>
       <c r="E1699" t="s">
-        <v>334</v>
+        <v>337</v>
       </c>
       <c r="F1699" s="1">
         <v>0</v>
       </c>
       <c r="G1699" s="1">
-        <v>22800</v>
+        <v>1584</v>
       </c>
       <c r="H1699" s="1">
         <v>0</v>
       </c>
       <c r="I1699" s="1">
-        <v>22800</v>
+        <v>1584</v>
       </c>
     </row>
     <row r="1700" spans="1:9" ht="12.75">
@@ -50846,19 +50846,19 @@
         <v>307</v>
       </c>
       <c r="E1700" t="s">
-        <v>335</v>
+        <v>338</v>
       </c>
       <c r="F1700" s="1">
         <v>0</v>
       </c>
       <c r="G1700" s="1">
-        <v>12631</v>
+        <v>10660</v>
       </c>
       <c r="H1700" s="1">
         <v>0</v>
       </c>
       <c r="I1700" s="1">
-        <v>12631</v>
+        <v>10660</v>
       </c>
     </row>
     <row r="1701" spans="1:9" ht="12.75">
@@ -50875,19 +50875,19 @@
         <v>307</v>
       </c>
       <c r="E1701" t="s">
-        <v>336</v>
+        <v>339</v>
       </c>
       <c r="F1701" s="1">
         <v>0</v>
       </c>
       <c r="G1701" s="1">
-        <v>179</v>
+        <v>154499</v>
       </c>
       <c r="H1701" s="1">
-        <v>0</v>
+        <v>154499</v>
       </c>
       <c r="I1701" s="1">
-        <v>179</v>
+        <v>0</v>
       </c>
     </row>
     <row r="1702" spans="1:9" ht="12.75">
@@ -50904,19 +50904,19 @@
         <v>307</v>
       </c>
       <c r="E1702" t="s">
-        <v>337</v>
+        <v>340</v>
       </c>
       <c r="F1702" s="1">
         <v>0</v>
       </c>
       <c r="G1702" s="1">
-        <v>1584</v>
+        <v>249</v>
       </c>
       <c r="H1702" s="1">
         <v>0</v>
       </c>
       <c r="I1702" s="1">
-        <v>1584</v>
+        <v>249</v>
       </c>
     </row>
     <row r="1703" spans="1:9" ht="12.75">
@@ -50933,19 +50933,19 @@
         <v>307</v>
       </c>
       <c r="E1703" t="s">
-        <v>338</v>
+        <v>341</v>
       </c>
       <c r="F1703" s="1">
         <v>0</v>
       </c>
       <c r="G1703" s="1">
-        <v>10660</v>
+        <v>375</v>
       </c>
       <c r="H1703" s="1">
         <v>0</v>
       </c>
       <c r="I1703" s="1">
-        <v>10660</v>
+        <v>375</v>
       </c>
     </row>
     <row r="1704" spans="1:9" ht="12.75">
@@ -50962,19 +50962,19 @@
         <v>307</v>
       </c>
       <c r="E1704" t="s">
-        <v>339</v>
+        <v>342</v>
       </c>
       <c r="F1704" s="1">
         <v>0</v>
       </c>
       <c r="G1704" s="1">
-        <v>154499</v>
+        <v>667</v>
       </c>
       <c r="H1704" s="1">
-        <v>154499</v>
+        <v>0</v>
       </c>
       <c r="I1704" s="1">
-        <v>0</v>
+        <v>667</v>
       </c>
     </row>
     <row r="1705" spans="1:9" ht="12.75">
@@ -50988,22 +50988,22 @@
         <v>105</v>
       </c>
       <c r="D1705" t="s">
-        <v>307</v>
+        <v>228</v>
       </c>
       <c r="E1705" t="s">
-        <v>340</v>
+        <v>348</v>
       </c>
       <c r="F1705" s="1">
         <v>0</v>
       </c>
       <c r="G1705" s="1">
-        <v>249</v>
+        <v>121502</v>
       </c>
       <c r="H1705" s="1">
         <v>0</v>
       </c>
       <c r="I1705" s="1">
-        <v>249</v>
+        <v>121502</v>
       </c>
     </row>
     <row r="1706" spans="1:9" ht="12.75">
@@ -51017,22 +51017,22 @@
         <v>105</v>
       </c>
       <c r="D1706" t="s">
-        <v>307</v>
+        <v>233</v>
       </c>
       <c r="E1706" t="s">
-        <v>341</v>
+        <v>330</v>
       </c>
       <c r="F1706" s="1">
         <v>0</v>
       </c>
       <c r="G1706" s="1">
-        <v>375</v>
+        <v>3500</v>
       </c>
       <c r="H1706" s="1">
         <v>0</v>
       </c>
       <c r="I1706" s="1">
-        <v>375</v>
+        <v>3500</v>
       </c>
     </row>
     <row r="1707" spans="1:9" ht="12.75">
@@ -51046,22 +51046,22 @@
         <v>105</v>
       </c>
       <c r="D1707" t="s">
-        <v>307</v>
+        <v>234</v>
       </c>
       <c r="E1707" t="s">
-        <v>342</v>
+        <v>343</v>
       </c>
       <c r="F1707" s="1">
         <v>0</v>
       </c>
       <c r="G1707" s="1">
-        <v>667</v>
+        <v>9000</v>
       </c>
       <c r="H1707" s="1">
         <v>0</v>
       </c>
       <c r="I1707" s="1">
-        <v>667</v>
+        <v>9000</v>
       </c>
     </row>
     <row r="1708" spans="1:9" ht="12.75">
@@ -51075,22 +51075,22 @@
         <v>105</v>
       </c>
       <c r="D1708" t="s">
-        <v>228</v>
+        <v>234</v>
       </c>
       <c r="E1708" t="s">
-        <v>348</v>
+        <v>339</v>
       </c>
       <c r="F1708" s="1">
         <v>0</v>
       </c>
       <c r="G1708" s="1">
-        <v>121502</v>
+        <v>516448</v>
       </c>
       <c r="H1708" s="1">
         <v>0</v>
       </c>
       <c r="I1708" s="1">
-        <v>121502</v>
+        <v>516448</v>
       </c>
     </row>
     <row r="1709" spans="1:9" ht="12.75">
@@ -51104,22 +51104,22 @@
         <v>105</v>
       </c>
       <c r="D1709" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="E1709" t="s">
-        <v>330</v>
+        <v>244</v>
       </c>
       <c r="F1709" s="1">
         <v>0</v>
       </c>
       <c r="G1709" s="1">
-        <v>3500</v>
+        <v>853156</v>
       </c>
       <c r="H1709" s="1">
         <v>0</v>
       </c>
       <c r="I1709" s="1">
-        <v>3500</v>
+        <v>853156</v>
       </c>
     </row>
     <row r="1710" spans="1:9" ht="12.75">
@@ -51133,22 +51133,22 @@
         <v>105</v>
       </c>
       <c r="D1710" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="E1710" t="s">
-        <v>343</v>
+        <v>351</v>
       </c>
       <c r="F1710" s="1">
         <v>0</v>
       </c>
       <c r="G1710" s="1">
-        <v>9000</v>
+        <v>1317706</v>
       </c>
       <c r="H1710" s="1">
         <v>0</v>
       </c>
       <c r="I1710" s="1">
-        <v>9000</v>
+        <v>1317706</v>
       </c>
     </row>
     <row r="1711" spans="1:9" ht="12.75">
@@ -51162,22 +51162,22 @@
         <v>105</v>
       </c>
       <c r="D1711" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="E1711" t="s">
-        <v>339</v>
+        <v>352</v>
       </c>
       <c r="F1711" s="1">
         <v>0</v>
       </c>
       <c r="G1711" s="1">
-        <v>516448</v>
+        <v>3665552</v>
       </c>
       <c r="H1711" s="1">
         <v>0</v>
       </c>
       <c r="I1711" s="1">
-        <v>516448</v>
+        <v>3665552</v>
       </c>
     </row>
     <row r="1712" spans="1:9" ht="12.75">
@@ -51194,19 +51194,19 @@
         <v>235</v>
       </c>
       <c r="E1712" t="s">
-        <v>244</v>
+        <v>353</v>
       </c>
       <c r="F1712" s="1">
         <v>0</v>
       </c>
       <c r="G1712" s="1">
-        <v>853156</v>
+        <v>2999088</v>
       </c>
       <c r="H1712" s="1">
         <v>0</v>
       </c>
       <c r="I1712" s="1">
-        <v>853156</v>
+        <v>2999088</v>
       </c>
     </row>
     <row r="1713" spans="1:9" ht="12.75">
@@ -51223,19 +51223,19 @@
         <v>235</v>
       </c>
       <c r="E1713" t="s">
-        <v>351</v>
+        <v>354</v>
       </c>
       <c r="F1713" s="1">
         <v>0</v>
       </c>
       <c r="G1713" s="1">
-        <v>1317706</v>
+        <v>709534</v>
       </c>
       <c r="H1713" s="1">
         <v>0</v>
       </c>
       <c r="I1713" s="1">
-        <v>1317706</v>
+        <v>709534</v>
       </c>
     </row>
     <row r="1714" spans="1:9" ht="12.75">
@@ -51249,22 +51249,22 @@
         <v>105</v>
       </c>
       <c r="D1714" t="s">
-        <v>235</v>
+        <v>237</v>
       </c>
       <c r="E1714" t="s">
-        <v>352</v>
+        <v>330</v>
       </c>
       <c r="F1714" s="1">
         <v>0</v>
       </c>
       <c r="G1714" s="1">
-        <v>3665552</v>
+        <v>31500</v>
       </c>
       <c r="H1714" s="1">
         <v>0</v>
       </c>
       <c r="I1714" s="1">
-        <v>3665552</v>
+        <v>31500</v>
       </c>
     </row>
     <row r="1715" spans="1:9" ht="12.75">
@@ -51278,22 +51278,22 @@
         <v>105</v>
       </c>
       <c r="D1715" t="s">
-        <v>235</v>
+        <v>238</v>
       </c>
       <c r="E1715" t="s">
-        <v>353</v>
+        <v>329</v>
       </c>
       <c r="F1715" s="1">
         <v>0</v>
       </c>
       <c r="G1715" s="1">
-        <v>2999088</v>
+        <v>212400</v>
       </c>
       <c r="H1715" s="1">
         <v>0</v>
       </c>
       <c r="I1715" s="1">
-        <v>2999088</v>
+        <v>212400</v>
       </c>
     </row>
     <row r="1716" spans="1:9" ht="12.75">
@@ -51307,22 +51307,22 @@
         <v>105</v>
       </c>
       <c r="D1716" t="s">
-        <v>235</v>
+        <v>238</v>
       </c>
       <c r="E1716" t="s">
-        <v>354</v>
+        <v>330</v>
       </c>
       <c r="F1716" s="1">
         <v>0</v>
       </c>
       <c r="G1716" s="1">
-        <v>709534</v>
+        <v>577360</v>
       </c>
       <c r="H1716" s="1">
         <v>0</v>
       </c>
       <c r="I1716" s="1">
-        <v>709534</v>
+        <v>577360</v>
       </c>
     </row>
     <row r="1717" spans="1:9" ht="12.75">
@@ -51336,22 +51336,22 @@
         <v>105</v>
       </c>
       <c r="D1717" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="E1717" t="s">
-        <v>330</v>
+        <v>331</v>
       </c>
       <c r="F1717" s="1">
         <v>0</v>
       </c>
       <c r="G1717" s="1">
-        <v>31500</v>
+        <v>518969</v>
       </c>
       <c r="H1717" s="1">
         <v>0</v>
       </c>
       <c r="I1717" s="1">
-        <v>31500</v>
+        <v>518969</v>
       </c>
     </row>
     <row r="1718" spans="1:9" ht="12.75">
@@ -51368,19 +51368,19 @@
         <v>238</v>
       </c>
       <c r="E1718" t="s">
-        <v>329</v>
+        <v>334</v>
       </c>
       <c r="F1718" s="1">
         <v>0</v>
       </c>
       <c r="G1718" s="1">
-        <v>212400</v>
+        <v>271070</v>
       </c>
       <c r="H1718" s="1">
         <v>0</v>
       </c>
       <c r="I1718" s="1">
-        <v>212400</v>
+        <v>271070</v>
       </c>
     </row>
     <row r="1719" spans="1:9" ht="12.75">
@@ -51397,19 +51397,19 @@
         <v>238</v>
       </c>
       <c r="E1719" t="s">
-        <v>330</v>
+        <v>335</v>
       </c>
       <c r="F1719" s="1">
         <v>0</v>
       </c>
       <c r="G1719" s="1">
-        <v>577360</v>
+        <v>137184</v>
       </c>
       <c r="H1719" s="1">
         <v>0</v>
       </c>
       <c r="I1719" s="1">
-        <v>577360</v>
+        <v>137184</v>
       </c>
     </row>
     <row r="1720" spans="1:9" ht="12.75">
@@ -51426,19 +51426,19 @@
         <v>238</v>
       </c>
       <c r="E1720" t="s">
-        <v>331</v>
+        <v>337</v>
       </c>
       <c r="F1720" s="1">
         <v>0</v>
       </c>
       <c r="G1720" s="1">
-        <v>518969</v>
+        <v>91456</v>
       </c>
       <c r="H1720" s="1">
         <v>0</v>
       </c>
       <c r="I1720" s="1">
-        <v>518969</v>
+        <v>91456</v>
       </c>
     </row>
     <row r="1721" spans="1:9" ht="12.75">
@@ -51455,19 +51455,19 @@
         <v>238</v>
       </c>
       <c r="E1721" t="s">
-        <v>334</v>
+        <v>352</v>
       </c>
       <c r="F1721" s="1">
         <v>0</v>
       </c>
       <c r="G1721" s="1">
-        <v>271070</v>
+        <v>8275</v>
       </c>
       <c r="H1721" s="1">
         <v>0</v>
       </c>
       <c r="I1721" s="1">
-        <v>271070</v>
+        <v>8275</v>
       </c>
     </row>
     <row r="1722" spans="1:9" ht="12.75">
@@ -51484,19 +51484,19 @@
         <v>238</v>
       </c>
       <c r="E1722" t="s">
-        <v>335</v>
+        <v>345</v>
       </c>
       <c r="F1722" s="1">
         <v>0</v>
       </c>
       <c r="G1722" s="1">
-        <v>137184</v>
+        <v>104725</v>
       </c>
       <c r="H1722" s="1">
         <v>0</v>
       </c>
       <c r="I1722" s="1">
-        <v>137184</v>
+        <v>104725</v>
       </c>
     </row>
     <row r="1723" spans="1:9" ht="12.75">
@@ -51510,22 +51510,22 @@
         <v>105</v>
       </c>
       <c r="D1723" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="E1723" t="s">
-        <v>337</v>
+        <v>330</v>
       </c>
       <c r="F1723" s="1">
         <v>0</v>
       </c>
       <c r="G1723" s="1">
-        <v>91456</v>
+        <v>8770</v>
       </c>
       <c r="H1723" s="1">
         <v>0</v>
       </c>
       <c r="I1723" s="1">
-        <v>91456</v>
+        <v>8770</v>
       </c>
     </row>
     <row r="1724" spans="1:9" ht="12.75">
@@ -51539,22 +51539,22 @@
         <v>105</v>
       </c>
       <c r="D1724" t="s">
-        <v>238</v>
+        <v>240</v>
       </c>
       <c r="E1724" t="s">
-        <v>352</v>
+        <v>330</v>
       </c>
       <c r="F1724" s="1">
         <v>0</v>
       </c>
       <c r="G1724" s="1">
-        <v>8275</v>
+        <v>62919.34</v>
       </c>
       <c r="H1724" s="1">
         <v>0</v>
       </c>
       <c r="I1724" s="1">
-        <v>8275</v>
+        <v>62919.34</v>
       </c>
     </row>
     <row r="1725" spans="1:9" ht="12.75">
@@ -51568,22 +51568,22 @@
         <v>105</v>
       </c>
       <c r="D1725" t="s">
-        <v>238</v>
+        <v>241</v>
       </c>
       <c r="E1725" t="s">
-        <v>345</v>
+        <v>13</v>
       </c>
       <c r="F1725" s="1">
         <v>0</v>
       </c>
       <c r="G1725" s="1">
-        <v>104725</v>
+        <v>1</v>
       </c>
       <c r="H1725" s="1">
-        <v>0</v>
+        <v>12.20</v>
       </c>
       <c r="I1725" s="1">
-        <v>104725</v>
+        <v>-11.20</v>
       </c>
     </row>
     <row r="1726" spans="1:9" ht="12.75">
@@ -51597,22 +51597,22 @@
         <v>105</v>
       </c>
       <c r="D1726" t="s">
-        <v>239</v>
+        <v>243</v>
       </c>
       <c r="E1726" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="F1726" s="1">
         <v>0</v>
       </c>
       <c r="G1726" s="1">
-        <v>8770</v>
+        <v>8760</v>
       </c>
       <c r="H1726" s="1">
         <v>0</v>
       </c>
       <c r="I1726" s="1">
-        <v>8770</v>
+        <v>8760</v>
       </c>
     </row>
     <row r="1727" spans="1:9" ht="12.75">
@@ -51626,22 +51626,22 @@
         <v>105</v>
       </c>
       <c r="D1727" t="s">
-        <v>240</v>
+        <v>243</v>
       </c>
       <c r="E1727" t="s">
-        <v>330</v>
+        <v>331</v>
       </c>
       <c r="F1727" s="1">
         <v>0</v>
       </c>
       <c r="G1727" s="1">
-        <v>62919.34</v>
+        <v>1205693</v>
       </c>
       <c r="H1727" s="1">
         <v>0</v>
       </c>
       <c r="I1727" s="1">
-        <v>62919.34</v>
+        <v>1205693</v>
       </c>
     </row>
     <row r="1728" spans="1:9" ht="12.75">
@@ -51655,22 +51655,22 @@
         <v>105</v>
       </c>
       <c r="D1728" t="s">
-        <v>241</v>
+        <v>243</v>
       </c>
       <c r="E1728" t="s">
-        <v>13</v>
+        <v>334</v>
       </c>
       <c r="F1728" s="1">
         <v>0</v>
       </c>
       <c r="G1728" s="1">
-        <v>1</v>
+        <v>117363390</v>
       </c>
       <c r="H1728" s="1">
-        <v>12.20</v>
+        <v>0</v>
       </c>
       <c r="I1728" s="1">
-        <v>-11.20</v>
+        <v>117363390</v>
       </c>
     </row>
     <row r="1729" spans="1:9" ht="12.75">
@@ -51687,19 +51687,19 @@
         <v>243</v>
       </c>
       <c r="E1729" t="s">
-        <v>329</v>
+        <v>335</v>
       </c>
       <c r="F1729" s="1">
         <v>0</v>
       </c>
       <c r="G1729" s="1">
-        <v>8760</v>
+        <v>10830040</v>
       </c>
       <c r="H1729" s="1">
         <v>0</v>
       </c>
       <c r="I1729" s="1">
-        <v>8760</v>
+        <v>10830040</v>
       </c>
     </row>
     <row r="1730" spans="1:9" ht="12.75">
@@ -51716,19 +51716,19 @@
         <v>243</v>
       </c>
       <c r="E1730" t="s">
-        <v>331</v>
+        <v>338</v>
       </c>
       <c r="F1730" s="1">
         <v>0</v>
       </c>
       <c r="G1730" s="1">
-        <v>1205693</v>
+        <v>5015000</v>
       </c>
       <c r="H1730" s="1">
         <v>0</v>
       </c>
       <c r="I1730" s="1">
-        <v>1205693</v>
+        <v>5015000</v>
       </c>
     </row>
     <row r="1731" spans="1:9" ht="12.75">
@@ -51745,19 +51745,19 @@
         <v>243</v>
       </c>
       <c r="E1731" t="s">
-        <v>334</v>
+        <v>341</v>
       </c>
       <c r="F1731" s="1">
         <v>0</v>
       </c>
       <c r="G1731" s="1">
-        <v>117363390</v>
+        <v>33458322</v>
       </c>
       <c r="H1731" s="1">
         <v>0</v>
       </c>
       <c r="I1731" s="1">
-        <v>117363390</v>
+        <v>33458322</v>
       </c>
     </row>
     <row r="1732" spans="1:9" ht="12.75">
@@ -51774,19 +51774,19 @@
         <v>243</v>
       </c>
       <c r="E1732" t="s">
-        <v>335</v>
+        <v>346</v>
       </c>
       <c r="F1732" s="1">
         <v>0</v>
       </c>
       <c r="G1732" s="1">
-        <v>10830040</v>
+        <v>1194533</v>
       </c>
       <c r="H1732" s="1">
         <v>0</v>
       </c>
       <c r="I1732" s="1">
-        <v>10830040</v>
+        <v>1194533</v>
       </c>
     </row>
     <row r="1733" spans="1:9" ht="12.75">
@@ -51800,22 +51800,22 @@
         <v>105</v>
       </c>
       <c r="D1733" t="s">
-        <v>243</v>
+        <v>246</v>
       </c>
       <c r="E1733" t="s">
-        <v>338</v>
+        <v>331</v>
       </c>
       <c r="F1733" s="1">
         <v>0</v>
       </c>
       <c r="G1733" s="1">
-        <v>5015000</v>
+        <v>31481</v>
       </c>
       <c r="H1733" s="1">
         <v>0</v>
       </c>
       <c r="I1733" s="1">
-        <v>5015000</v>
+        <v>31481</v>
       </c>
     </row>
     <row r="1734" spans="1:9" ht="12.75">
@@ -51829,22 +51829,22 @@
         <v>105</v>
       </c>
       <c r="D1734" t="s">
-        <v>243</v>
+        <v>246</v>
       </c>
       <c r="E1734" t="s">
-        <v>341</v>
+        <v>332</v>
       </c>
       <c r="F1734" s="1">
         <v>0</v>
       </c>
       <c r="G1734" s="1">
-        <v>33458322</v>
+        <v>6638</v>
       </c>
       <c r="H1734" s="1">
         <v>0</v>
       </c>
       <c r="I1734" s="1">
-        <v>33458322</v>
+        <v>6638</v>
       </c>
     </row>
     <row r="1735" spans="1:9" ht="12.75">
@@ -51858,22 +51858,22 @@
         <v>105</v>
       </c>
       <c r="D1735" t="s">
-        <v>243</v>
+        <v>246</v>
       </c>
       <c r="E1735" t="s">
-        <v>346</v>
+        <v>355</v>
       </c>
       <c r="F1735" s="1">
         <v>0</v>
       </c>
       <c r="G1735" s="1">
-        <v>1194533</v>
+        <v>7140</v>
       </c>
       <c r="H1735" s="1">
         <v>0</v>
       </c>
       <c r="I1735" s="1">
-        <v>1194533</v>
+        <v>7140</v>
       </c>
     </row>
     <row r="1736" spans="1:9" ht="12.75">
@@ -51890,19 +51890,19 @@
         <v>246</v>
       </c>
       <c r="E1736" t="s">
-        <v>331</v>
+        <v>338</v>
       </c>
       <c r="F1736" s="1">
         <v>0</v>
       </c>
       <c r="G1736" s="1">
-        <v>31481</v>
+        <v>41204</v>
       </c>
       <c r="H1736" s="1">
         <v>0</v>
       </c>
       <c r="I1736" s="1">
-        <v>31481</v>
+        <v>41204</v>
       </c>
     </row>
     <row r="1737" spans="1:9" ht="12.75">
@@ -51916,22 +51916,22 @@
         <v>105</v>
       </c>
       <c r="D1737" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="E1737" t="s">
-        <v>332</v>
+        <v>329</v>
       </c>
       <c r="F1737" s="1">
         <v>0</v>
       </c>
       <c r="G1737" s="1">
-        <v>6638</v>
+        <v>77571</v>
       </c>
       <c r="H1737" s="1">
         <v>0</v>
       </c>
       <c r="I1737" s="1">
-        <v>6638</v>
+        <v>77571</v>
       </c>
     </row>
     <row r="1738" spans="1:9" ht="12.75">
@@ -51945,22 +51945,22 @@
         <v>105</v>
       </c>
       <c r="D1738" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="E1738" t="s">
-        <v>355</v>
+        <v>330</v>
       </c>
       <c r="F1738" s="1">
         <v>0</v>
       </c>
       <c r="G1738" s="1">
-        <v>7140</v>
+        <v>1513824</v>
       </c>
       <c r="H1738" s="1">
         <v>0</v>
       </c>
       <c r="I1738" s="1">
-        <v>7140</v>
+        <v>1513824</v>
       </c>
     </row>
     <row r="1739" spans="1:9" ht="12.75">
@@ -51974,22 +51974,22 @@
         <v>105</v>
       </c>
       <c r="D1739" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="E1739" t="s">
-        <v>338</v>
+        <v>332</v>
       </c>
       <c r="F1739" s="1">
         <v>0</v>
       </c>
       <c r="G1739" s="1">
-        <v>41204</v>
+        <v>22538</v>
       </c>
       <c r="H1739" s="1">
         <v>0</v>
       </c>
       <c r="I1739" s="1">
-        <v>41204</v>
+        <v>22538</v>
       </c>
     </row>
     <row r="1740" spans="1:9" ht="12.75">
@@ -52003,22 +52003,22 @@
         <v>105</v>
       </c>
       <c r="D1740" t="s">
-        <v>247</v>
+        <v>249</v>
       </c>
       <c r="E1740" t="s">
-        <v>329</v>
+        <v>331</v>
       </c>
       <c r="F1740" s="1">
         <v>0</v>
       </c>
       <c r="G1740" s="1">
-        <v>77571</v>
+        <v>9676</v>
       </c>
       <c r="H1740" s="1">
         <v>0</v>
       </c>
       <c r="I1740" s="1">
-        <v>77571</v>
+        <v>9676</v>
       </c>
     </row>
     <row r="1741" spans="1:9" ht="12.75">
@@ -52032,22 +52032,22 @@
         <v>105</v>
       </c>
       <c r="D1741" t="s">
-        <v>247</v>
+        <v>250</v>
       </c>
       <c r="E1741" t="s">
-        <v>330</v>
+        <v>13</v>
       </c>
       <c r="F1741" s="1">
         <v>0</v>
       </c>
       <c r="G1741" s="1">
-        <v>1513824</v>
+        <v>0</v>
       </c>
       <c r="H1741" s="1">
-        <v>0</v>
+        <v>13663</v>
       </c>
       <c r="I1741" s="1">
-        <v>1513824</v>
+        <v>-13663</v>
       </c>
     </row>
     <row r="1742" spans="1:9" ht="12.75">
@@ -52061,22 +52061,22 @@
         <v>105</v>
       </c>
       <c r="D1742" t="s">
-        <v>247</v>
+        <v>250</v>
       </c>
       <c r="E1742" t="s">
-        <v>332</v>
+        <v>329</v>
       </c>
       <c r="F1742" s="1">
         <v>0</v>
       </c>
       <c r="G1742" s="1">
-        <v>22538</v>
+        <v>3353166</v>
       </c>
       <c r="H1742" s="1">
         <v>0</v>
       </c>
       <c r="I1742" s="1">
-        <v>22538</v>
+        <v>3353166</v>
       </c>
     </row>
     <row r="1743" spans="1:9" ht="12.75">
@@ -52090,22 +52090,22 @@
         <v>105</v>
       </c>
       <c r="D1743" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="E1743" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="F1743" s="1">
         <v>0</v>
       </c>
       <c r="G1743" s="1">
-        <v>9676</v>
+        <v>662779</v>
       </c>
       <c r="H1743" s="1">
         <v>0</v>
       </c>
       <c r="I1743" s="1">
-        <v>9676</v>
+        <v>662779</v>
       </c>
     </row>
     <row r="1744" spans="1:9" ht="12.75">
@@ -52122,19 +52122,19 @@
         <v>250</v>
       </c>
       <c r="E1744" t="s">
-        <v>13</v>
+        <v>331</v>
       </c>
       <c r="F1744" s="1">
         <v>0</v>
       </c>
       <c r="G1744" s="1">
-        <v>0</v>
+        <v>31417864</v>
       </c>
       <c r="H1744" s="1">
-        <v>13663</v>
+        <v>0</v>
       </c>
       <c r="I1744" s="1">
-        <v>-13663</v>
+        <v>31417864</v>
       </c>
     </row>
     <row r="1745" spans="1:9" ht="12.75">
@@ -52151,19 +52151,19 @@
         <v>250</v>
       </c>
       <c r="E1745" t="s">
-        <v>329</v>
+        <v>332</v>
       </c>
       <c r="F1745" s="1">
         <v>0</v>
       </c>
       <c r="G1745" s="1">
-        <v>3353166</v>
+        <v>2664907</v>
       </c>
       <c r="H1745" s="1">
         <v>0</v>
       </c>
       <c r="I1745" s="1">
-        <v>3353166</v>
+        <v>2664907</v>
       </c>
     </row>
     <row r="1746" spans="1:9" ht="12.75">
@@ -52180,19 +52180,19 @@
         <v>250</v>
       </c>
       <c r="E1746" t="s">
-        <v>330</v>
+        <v>333</v>
       </c>
       <c r="F1746" s="1">
         <v>0</v>
       </c>
       <c r="G1746" s="1">
-        <v>662779</v>
+        <v>2021829</v>
       </c>
       <c r="H1746" s="1">
         <v>0</v>
       </c>
       <c r="I1746" s="1">
-        <v>662779</v>
+        <v>2021829</v>
       </c>
     </row>
     <row r="1747" spans="1:9" ht="12.75">
@@ -52209,19 +52209,19 @@
         <v>250</v>
       </c>
       <c r="E1747" t="s">
-        <v>331</v>
+        <v>334</v>
       </c>
       <c r="F1747" s="1">
         <v>0</v>
       </c>
       <c r="G1747" s="1">
-        <v>31417864</v>
+        <v>14946353</v>
       </c>
       <c r="H1747" s="1">
         <v>0</v>
       </c>
       <c r="I1747" s="1">
-        <v>31417864</v>
+        <v>14946353</v>
       </c>
     </row>
     <row r="1748" spans="1:9" ht="12.75">
@@ -52238,19 +52238,19 @@
         <v>250</v>
       </c>
       <c r="E1748" t="s">
-        <v>332</v>
+        <v>335</v>
       </c>
       <c r="F1748" s="1">
         <v>0</v>
       </c>
       <c r="G1748" s="1">
-        <v>2664907</v>
+        <v>5986158</v>
       </c>
       <c r="H1748" s="1">
         <v>0</v>
       </c>
       <c r="I1748" s="1">
-        <v>2664907</v>
+        <v>5986158</v>
       </c>
     </row>
     <row r="1749" spans="1:9" ht="12.75">
@@ -52267,19 +52267,19 @@
         <v>250</v>
       </c>
       <c r="E1749" t="s">
-        <v>333</v>
+        <v>336</v>
       </c>
       <c r="F1749" s="1">
         <v>0</v>
       </c>
       <c r="G1749" s="1">
-        <v>2021829</v>
+        <v>30819</v>
       </c>
       <c r="H1749" s="1">
         <v>0</v>
       </c>
       <c r="I1749" s="1">
-        <v>2021829</v>
+        <v>30819</v>
       </c>
     </row>
     <row r="1750" spans="1:9" ht="12.75">
@@ -52296,19 +52296,19 @@
         <v>250</v>
       </c>
       <c r="E1750" t="s">
-        <v>334</v>
+        <v>337</v>
       </c>
       <c r="F1750" s="1">
         <v>0</v>
       </c>
       <c r="G1750" s="1">
-        <v>14946353</v>
+        <v>1516559</v>
       </c>
       <c r="H1750" s="1">
         <v>0</v>
       </c>
       <c r="I1750" s="1">
-        <v>14946353</v>
+        <v>1516559</v>
       </c>
     </row>
     <row r="1751" spans="1:9" ht="12.75">
@@ -52325,19 +52325,19 @@
         <v>250</v>
       </c>
       <c r="E1751" t="s">
-        <v>335</v>
+        <v>338</v>
       </c>
       <c r="F1751" s="1">
         <v>0</v>
       </c>
       <c r="G1751" s="1">
-        <v>5986158</v>
+        <v>3492740</v>
       </c>
       <c r="H1751" s="1">
         <v>0</v>
       </c>
       <c r="I1751" s="1">
-        <v>5986158</v>
+        <v>3492740</v>
       </c>
     </row>
     <row r="1752" spans="1:9" ht="12.75">
@@ -52354,19 +52354,19 @@
         <v>250</v>
       </c>
       <c r="E1752" t="s">
-        <v>336</v>
+        <v>339</v>
       </c>
       <c r="F1752" s="1">
         <v>0</v>
       </c>
       <c r="G1752" s="1">
-        <v>30819</v>
+        <v>75917498</v>
       </c>
       <c r="H1752" s="1">
-        <v>0</v>
+        <v>75917498</v>
       </c>
       <c r="I1752" s="1">
-        <v>30819</v>
+        <v>0</v>
       </c>
     </row>
     <row r="1753" spans="1:9" ht="12.75">
@@ -52383,19 +52383,19 @@
         <v>250</v>
       </c>
       <c r="E1753" t="s">
-        <v>337</v>
+        <v>340</v>
       </c>
       <c r="F1753" s="1">
         <v>0</v>
       </c>
       <c r="G1753" s="1">
-        <v>1516559</v>
+        <v>747484</v>
       </c>
       <c r="H1753" s="1">
         <v>0</v>
       </c>
       <c r="I1753" s="1">
-        <v>1516559</v>
+        <v>747484</v>
       </c>
     </row>
     <row r="1754" spans="1:9" ht="12.75">
@@ -52412,19 +52412,19 @@
         <v>250</v>
       </c>
       <c r="E1754" t="s">
-        <v>338</v>
+        <v>341</v>
       </c>
       <c r="F1754" s="1">
         <v>0</v>
       </c>
       <c r="G1754" s="1">
-        <v>3492740</v>
+        <v>1826516</v>
       </c>
       <c r="H1754" s="1">
         <v>0</v>
       </c>
       <c r="I1754" s="1">
-        <v>3492740</v>
+        <v>1826516</v>
       </c>
     </row>
     <row r="1755" spans="1:9" ht="12.75">
@@ -52441,19 +52441,19 @@
         <v>250</v>
       </c>
       <c r="E1755" t="s">
-        <v>339</v>
+        <v>342</v>
       </c>
       <c r="F1755" s="1">
         <v>0</v>
       </c>
       <c r="G1755" s="1">
-        <v>75917498</v>
+        <v>9827272</v>
       </c>
       <c r="H1755" s="1">
-        <v>75917498</v>
+        <v>0</v>
       </c>
       <c r="I1755" s="1">
-        <v>0</v>
+        <v>9827272</v>
       </c>
     </row>
     <row r="1756" spans="1:9" ht="12.75">
@@ -52467,22 +52467,22 @@
         <v>105</v>
       </c>
       <c r="D1756" t="s">
-        <v>250</v>
+        <v>253</v>
       </c>
       <c r="E1756" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
       <c r="F1756" s="1">
         <v>0</v>
       </c>
       <c r="G1756" s="1">
-        <v>747484</v>
+        <v>0</v>
       </c>
       <c r="H1756" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I1756" s="1">
-        <v>747484</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="1757" spans="1:9" ht="12.75">
@@ -52496,22 +52496,22 @@
         <v>105</v>
       </c>
       <c r="D1757" t="s">
-        <v>250</v>
+        <v>257</v>
       </c>
       <c r="E1757" t="s">
-        <v>341</v>
+        <v>331</v>
       </c>
       <c r="F1757" s="1">
         <v>0</v>
       </c>
       <c r="G1757" s="1">
-        <v>1826516</v>
+        <v>148184</v>
       </c>
       <c r="H1757" s="1">
         <v>0</v>
       </c>
       <c r="I1757" s="1">
-        <v>1826516</v>
+        <v>148184</v>
       </c>
     </row>
     <row r="1758" spans="1:9" ht="12.75">
@@ -52525,22 +52525,22 @@
         <v>105</v>
       </c>
       <c r="D1758" t="s">
-        <v>250</v>
+        <v>257</v>
       </c>
       <c r="E1758" t="s">
-        <v>342</v>
+        <v>334</v>
       </c>
       <c r="F1758" s="1">
         <v>0</v>
       </c>
       <c r="G1758" s="1">
-        <v>9827272</v>
+        <v>74092</v>
       </c>
       <c r="H1758" s="1">
         <v>0</v>
       </c>
       <c r="I1758" s="1">
-        <v>9827272</v>
+        <v>74092</v>
       </c>
     </row>
     <row r="1759" spans="1:9" ht="12.75">
@@ -52554,22 +52554,22 @@
         <v>105</v>
       </c>
       <c r="D1759" t="s">
-        <v>253</v>
+        <v>257</v>
       </c>
       <c r="E1759" t="s">
-        <v>339</v>
+        <v>335</v>
       </c>
       <c r="F1759" s="1">
         <v>0</v>
       </c>
       <c r="G1759" s="1">
-        <v>0</v>
+        <v>74092.80</v>
       </c>
       <c r="H1759" s="1">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I1759" s="1">
-        <v>-1</v>
+        <v>74092.80</v>
       </c>
     </row>
     <row r="1760" spans="1:9" ht="12.75">
@@ -52583,22 +52583,22 @@
         <v>105</v>
       </c>
       <c r="D1760" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="E1760" t="s">
-        <v>331</v>
+        <v>329</v>
       </c>
       <c r="F1760" s="1">
         <v>0</v>
       </c>
       <c r="G1760" s="1">
-        <v>148184</v>
+        <v>137490</v>
       </c>
       <c r="H1760" s="1">
         <v>0</v>
       </c>
       <c r="I1760" s="1">
-        <v>148184</v>
+        <v>137490</v>
       </c>
     </row>
     <row r="1761" spans="1:9" ht="12.75">
@@ -52612,22 +52612,22 @@
         <v>105</v>
       </c>
       <c r="D1761" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="E1761" t="s">
-        <v>334</v>
+        <v>330</v>
       </c>
       <c r="F1761" s="1">
         <v>0</v>
       </c>
       <c r="G1761" s="1">
-        <v>74092</v>
+        <v>305648</v>
       </c>
       <c r="H1761" s="1">
         <v>0</v>
       </c>
       <c r="I1761" s="1">
-        <v>74092</v>
+        <v>305648</v>
       </c>
     </row>
     <row r="1762" spans="1:9" ht="12.75">
@@ -52641,22 +52641,22 @@
         <v>105</v>
       </c>
       <c r="D1762" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="E1762" t="s">
-        <v>335</v>
+        <v>331</v>
       </c>
       <c r="F1762" s="1">
         <v>0</v>
       </c>
       <c r="G1762" s="1">
-        <v>74092.80</v>
+        <v>484</v>
       </c>
       <c r="H1762" s="1">
         <v>0</v>
       </c>
       <c r="I1762" s="1">
-        <v>74092.80</v>
+        <v>484</v>
       </c>
     </row>
     <row r="1763" spans="1:9" ht="12.75">
@@ -52670,22 +52670,22 @@
         <v>105</v>
       </c>
       <c r="D1763" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="E1763" t="s">
-        <v>329</v>
+        <v>339</v>
       </c>
       <c r="F1763" s="1">
         <v>0</v>
       </c>
       <c r="G1763" s="1">
-        <v>137490</v>
+        <v>24000</v>
       </c>
       <c r="H1763" s="1">
         <v>0</v>
       </c>
       <c r="I1763" s="1">
-        <v>137490</v>
+        <v>24000</v>
       </c>
     </row>
     <row r="1764" spans="1:9" ht="12.75">
@@ -52699,22 +52699,22 @@
         <v>105</v>
       </c>
       <c r="D1764" t="s">
-        <v>258</v>
+        <v>263</v>
       </c>
       <c r="E1764" t="s">
-        <v>330</v>
+        <v>331</v>
       </c>
       <c r="F1764" s="1">
         <v>0</v>
       </c>
       <c r="G1764" s="1">
-        <v>305648</v>
+        <v>1125720</v>
       </c>
       <c r="H1764" s="1">
         <v>0</v>
       </c>
       <c r="I1764" s="1">
-        <v>305648</v>
+        <v>1125720</v>
       </c>
     </row>
     <row r="1765" spans="1:9" ht="12.75">
@@ -52728,22 +52728,22 @@
         <v>105</v>
       </c>
       <c r="D1765" t="s">
-        <v>258</v>
+        <v>263</v>
       </c>
       <c r="E1765" t="s">
-        <v>331</v>
+        <v>338</v>
       </c>
       <c r="F1765" s="1">
         <v>0</v>
       </c>
       <c r="G1765" s="1">
-        <v>484</v>
+        <v>1125720</v>
       </c>
       <c r="H1765" s="1">
         <v>0</v>
       </c>
       <c r="I1765" s="1">
-        <v>484</v>
+        <v>1125720</v>
       </c>
     </row>
     <row r="1766" spans="1:9" ht="12.75">
@@ -52751,28 +52751,28 @@
         <v>312</v>
       </c>
       <c r="B1766" t="s">
-        <v>105</v>
+        <v>264</v>
       </c>
       <c r="C1766" t="s">
-        <v>105</v>
+        <v>264</v>
       </c>
       <c r="D1766" t="s">
-        <v>259</v>
+        <v>267</v>
       </c>
       <c r="E1766" t="s">
-        <v>339</v>
+        <v>13</v>
       </c>
       <c r="F1766" s="1">
         <v>0</v>
       </c>
       <c r="G1766" s="1">
-        <v>24000</v>
+        <v>0</v>
       </c>
       <c r="H1766" s="1">
-        <v>0</v>
+        <v>7351276</v>
       </c>
       <c r="I1766" s="1">
-        <v>24000</v>
+        <v>-7351276</v>
       </c>
     </row>
     <row r="1767" spans="1:9" ht="12.75">
@@ -52780,28 +52780,28 @@
         <v>312</v>
       </c>
       <c r="B1767" t="s">
-        <v>105</v>
+        <v>264</v>
       </c>
       <c r="C1767" t="s">
-        <v>105</v>
+        <v>264</v>
       </c>
       <c r="D1767" t="s">
-        <v>263</v>
+        <v>308</v>
       </c>
       <c r="E1767" t="s">
-        <v>331</v>
+        <v>13</v>
       </c>
       <c r="F1767" s="1">
         <v>0</v>
       </c>
       <c r="G1767" s="1">
-        <v>1125720</v>
+        <v>0</v>
       </c>
       <c r="H1767" s="1">
         <v>0</v>
       </c>
       <c r="I1767" s="1">
-        <v>1125720</v>
+        <v>0</v>
       </c>
     </row>
     <row r="1768" spans="1:9" ht="12.75">
@@ -52809,28 +52809,28 @@
         <v>312</v>
       </c>
       <c r="B1768" t="s">
-        <v>105</v>
+        <v>268</v>
       </c>
       <c r="C1768" t="s">
-        <v>105</v>
+        <v>269</v>
       </c>
       <c r="D1768" t="s">
-        <v>263</v>
+        <v>269</v>
       </c>
       <c r="E1768" t="s">
-        <v>338</v>
+        <v>13</v>
       </c>
       <c r="F1768" s="1">
-        <v>0</v>
+        <v>-5418882</v>
       </c>
       <c r="G1768" s="1">
-        <v>1125720</v>
+        <v>2.3231524567000002E8</v>
       </c>
       <c r="H1768" s="1">
-        <v>0</v>
+        <v>2.6244316570000005E8</v>
       </c>
       <c r="I1768" s="1">
-        <v>1125720</v>
+        <v>-3.554680203000003E7</v>
       </c>
     </row>
     <row r="1769" spans="1:9" ht="12.75">
@@ -52838,13 +52838,13 @@
         <v>312</v>
       </c>
       <c r="B1769" t="s">
-        <v>264</v>
+        <v>268</v>
       </c>
       <c r="C1769" t="s">
-        <v>264</v>
+        <v>273</v>
       </c>
       <c r="D1769" t="s">
-        <v>267</v>
+        <v>356</v>
       </c>
       <c r="E1769" t="s">
         <v>13</v>
@@ -52853,13 +52853,13 @@
         <v>0</v>
       </c>
       <c r="G1769" s="1">
-        <v>0</v>
+        <v>2274999</v>
       </c>
       <c r="H1769" s="1">
-        <v>7351276</v>
+        <v>5013786</v>
       </c>
       <c r="I1769" s="1">
-        <v>-7351276</v>
+        <v>-2738787</v>
       </c>
     </row>
     <row r="1770" spans="1:9" ht="12.75">
@@ -52867,28 +52867,28 @@
         <v>312</v>
       </c>
       <c r="B1770" t="s">
-        <v>264</v>
+        <v>268</v>
       </c>
       <c r="C1770" t="s">
-        <v>264</v>
+        <v>273</v>
       </c>
       <c r="D1770" t="s">
-        <v>308</v>
+        <v>278</v>
       </c>
       <c r="E1770" t="s">
         <v>13</v>
       </c>
       <c r="F1770" s="1">
-        <v>0</v>
+        <v>-22030149</v>
       </c>
       <c r="G1770" s="1">
         <v>0</v>
       </c>
       <c r="H1770" s="1">
-        <v>0</v>
+        <v>9.094276758399999E8</v>
       </c>
       <c r="I1770" s="1">
-        <v>0</v>
+        <v>-9.314578248399999E8</v>
       </c>
     </row>
     <row r="1771" spans="1:9" ht="12.75">
@@ -52899,25 +52899,25 @@
         <v>268</v>
       </c>
       <c r="C1771" t="s">
-        <v>269</v>
+        <v>273</v>
       </c>
       <c r="D1771" t="s">
-        <v>269</v>
+        <v>282</v>
       </c>
       <c r="E1771" t="s">
         <v>13</v>
       </c>
       <c r="F1771" s="1">
-        <v>-5418882</v>
+        <v>-14989</v>
       </c>
       <c r="G1771" s="1">
-        <v>2.3231524567000002E8</v>
+        <v>5380456</v>
       </c>
       <c r="H1771" s="1">
-        <v>2.6244316570000002E8</v>
+        <v>10165830</v>
       </c>
       <c r="I1771" s="1">
-        <v>-3.554680203E7</v>
+        <v>-4800363</v>
       </c>
     </row>
     <row r="1772" spans="1:9" ht="12.75">
@@ -52931,7 +52931,7 @@
         <v>273</v>
       </c>
       <c r="D1772" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="E1772" t="s">
         <v>13</v>
@@ -52940,13 +52940,13 @@
         <v>0</v>
       </c>
       <c r="G1772" s="1">
-        <v>2274999</v>
+        <v>2659661</v>
       </c>
       <c r="H1772" s="1">
-        <v>5013786</v>
+        <v>2659660</v>
       </c>
       <c r="I1772" s="1">
-        <v>-2738787</v>
+        <v>1</v>
       </c>
     </row>
     <row r="1773" spans="1:9" ht="12.75">
@@ -52960,22 +52960,22 @@
         <v>273</v>
       </c>
       <c r="D1773" t="s">
-        <v>278</v>
+        <v>286</v>
       </c>
       <c r="E1773" t="s">
         <v>13</v>
       </c>
       <c r="F1773" s="1">
-        <v>-22030149</v>
+        <v>0</v>
       </c>
       <c r="G1773" s="1">
         <v>0</v>
       </c>
       <c r="H1773" s="1">
-        <v>9.094276758399999E8</v>
+        <v>190424</v>
       </c>
       <c r="I1773" s="1">
-        <v>-9.314578248399999E8</v>
+        <v>-190424</v>
       </c>
     </row>
     <row r="1774" spans="1:9" ht="12.75">
@@ -52989,22 +52989,22 @@
         <v>273</v>
       </c>
       <c r="D1774" t="s">
-        <v>282</v>
+        <v>358</v>
       </c>
       <c r="E1774" t="s">
         <v>13</v>
       </c>
       <c r="F1774" s="1">
-        <v>-14989</v>
+        <v>0</v>
       </c>
       <c r="G1774" s="1">
-        <v>5380456</v>
+        <v>1966914</v>
       </c>
       <c r="H1774" s="1">
-        <v>10165830</v>
+        <v>1995881</v>
       </c>
       <c r="I1774" s="1">
-        <v>-4800363</v>
+        <v>-28967</v>
       </c>
     </row>
     <row r="1775" spans="1:9" ht="12.75">
@@ -53018,7 +53018,7 @@
         <v>273</v>
       </c>
       <c r="D1775" t="s">
-        <v>357</v>
+        <v>287</v>
       </c>
       <c r="E1775" t="s">
         <v>13</v>
@@ -53027,13 +53027,13 @@
         <v>0</v>
       </c>
       <c r="G1775" s="1">
-        <v>2659661</v>
+        <v>46090</v>
       </c>
       <c r="H1775" s="1">
-        <v>2659660</v>
+        <v>70730</v>
       </c>
       <c r="I1775" s="1">
-        <v>1</v>
+        <v>-24640</v>
       </c>
     </row>
     <row r="1776" spans="1:9" ht="12.75">
@@ -53047,7 +53047,7 @@
         <v>273</v>
       </c>
       <c r="D1776" t="s">
-        <v>286</v>
+        <v>288</v>
       </c>
       <c r="E1776" t="s">
         <v>13</v>
@@ -53056,13 +53056,13 @@
         <v>0</v>
       </c>
       <c r="G1776" s="1">
-        <v>0</v>
+        <v>840</v>
       </c>
       <c r="H1776" s="1">
-        <v>190424</v>
+        <v>416</v>
       </c>
       <c r="I1776" s="1">
-        <v>-190424</v>
+        <v>424</v>
       </c>
     </row>
     <row r="1777" spans="1:9" ht="12.75">
@@ -53076,7 +53076,7 @@
         <v>273</v>
       </c>
       <c r="D1777" t="s">
-        <v>358</v>
+        <v>289</v>
       </c>
       <c r="E1777" t="s">
         <v>13</v>
@@ -53085,13 +53085,13 @@
         <v>0</v>
       </c>
       <c r="G1777" s="1">
-        <v>1966914</v>
+        <v>4.65382019E7</v>
       </c>
       <c r="H1777" s="1">
-        <v>1995881</v>
+        <v>58379674</v>
       </c>
       <c r="I1777" s="1">
-        <v>-28967</v>
+        <v>-1.1841472100000001E7</v>
       </c>
     </row>
     <row r="1778" spans="1:9" ht="12.75">
@@ -53105,7 +53105,7 @@
         <v>273</v>
       </c>
       <c r="D1778" t="s">
-        <v>287</v>
+        <v>291</v>
       </c>
       <c r="E1778" t="s">
         <v>13</v>
@@ -53114,13 +53114,13 @@
         <v>0</v>
       </c>
       <c r="G1778" s="1">
-        <v>46090</v>
+        <v>37299</v>
       </c>
       <c r="H1778" s="1">
-        <v>70730</v>
+        <v>185786.20</v>
       </c>
       <c r="I1778" s="1">
-        <v>-24640</v>
+        <v>-148487.20</v>
       </c>
     </row>
     <row r="1779" spans="1:9" ht="12.75">
@@ -53134,7 +53134,7 @@
         <v>273</v>
       </c>
       <c r="D1779" t="s">
-        <v>288</v>
+        <v>292</v>
       </c>
       <c r="E1779" t="s">
         <v>13</v>
@@ -53143,13 +53143,13 @@
         <v>0</v>
       </c>
       <c r="G1779" s="1">
-        <v>840</v>
+        <v>90747</v>
       </c>
       <c r="H1779" s="1">
-        <v>416</v>
+        <v>498838.89999999997</v>
       </c>
       <c r="I1779" s="1">
-        <v>424</v>
+        <v>-408091.89999999997</v>
       </c>
     </row>
     <row r="1780" spans="1:9" ht="12.75">
@@ -53163,7 +53163,7 @@
         <v>273</v>
       </c>
       <c r="D1780" t="s">
-        <v>289</v>
+        <v>293</v>
       </c>
       <c r="E1780" t="s">
         <v>13</v>
@@ -53172,13 +53172,13 @@
         <v>0</v>
       </c>
       <c r="G1780" s="1">
-        <v>4.65382019E7</v>
+        <v>4109064</v>
       </c>
       <c r="H1780" s="1">
-        <v>58379674</v>
+        <v>1.186267109E7</v>
       </c>
       <c r="I1780" s="1">
-        <v>-1.1841472100000001E7</v>
+        <v>-7753607.09</v>
       </c>
     </row>
     <row r="1781" spans="1:9" ht="12.75">
@@ -53192,7 +53192,7 @@
         <v>273</v>
       </c>
       <c r="D1781" t="s">
-        <v>291</v>
+        <v>294</v>
       </c>
       <c r="E1781" t="s">
         <v>13</v>
@@ -53201,13 +53201,13 @@
         <v>0</v>
       </c>
       <c r="G1781" s="1">
-        <v>37299</v>
+        <v>1758542.24</v>
       </c>
       <c r="H1781" s="1">
-        <v>185786.20</v>
+        <v>1153027.74</v>
       </c>
       <c r="I1781" s="1">
-        <v>-148487.20</v>
+        <v>605514.50</v>
       </c>
     </row>
     <row r="1782" spans="1:9" ht="12.75">
@@ -53221,7 +53221,7 @@
         <v>273</v>
       </c>
       <c r="D1782" t="s">
-        <v>292</v>
+        <v>359</v>
       </c>
       <c r="E1782" t="s">
         <v>13</v>
@@ -53230,13 +53230,13 @@
         <v>0</v>
       </c>
       <c r="G1782" s="1">
-        <v>90747</v>
+        <v>8601440</v>
       </c>
       <c r="H1782" s="1">
-        <v>498838.89999999997</v>
+        <v>18873669</v>
       </c>
       <c r="I1782" s="1">
-        <v>-408091.89999999997</v>
+        <v>-10272229</v>
       </c>
     </row>
     <row r="1783" spans="1:9" ht="12.75">
@@ -53247,10 +53247,10 @@
         <v>268</v>
       </c>
       <c r="C1783" t="s">
-        <v>273</v>
+        <v>296</v>
       </c>
       <c r="D1783" t="s">
-        <v>293</v>
+        <v>297</v>
       </c>
       <c r="E1783" t="s">
         <v>13</v>
@@ -53259,13 +53259,13 @@
         <v>0</v>
       </c>
       <c r="G1783" s="1">
-        <v>4109064</v>
+        <v>2.2509215249E8</v>
       </c>
       <c r="H1783" s="1">
-        <v>1.186267109E7</v>
+        <v>2.2509215249E8</v>
       </c>
       <c r="I1783" s="1">
-        <v>-7753607.09</v>
+        <v>0</v>
       </c>
     </row>
     <row r="1784" spans="1:9" ht="12.75">
@@ -53276,10 +53276,10 @@
         <v>268</v>
       </c>
       <c r="C1784" t="s">
-        <v>273</v>
+        <v>296</v>
       </c>
       <c r="D1784" t="s">
-        <v>294</v>
+        <v>298</v>
       </c>
       <c r="E1784" t="s">
         <v>13</v>
@@ -53288,129 +53288,42 @@
         <v>0</v>
       </c>
       <c r="G1784" s="1">
-        <v>1758542.24</v>
+        <v>0</v>
       </c>
       <c r="H1784" s="1">
-        <v>1153027.74</v>
+        <v>8826219.66</v>
       </c>
       <c r="I1784" s="1">
-        <v>605514.50</v>
+        <v>-8826219.66</v>
       </c>
     </row>
     <row r="1785" spans="1:9" ht="12.75">
       <c r="A1785" t="s">
-        <v>312</v>
+        <v>360</v>
       </c>
       <c r="B1785" t="s">
-        <v>268</v>
+        <v>361</v>
       </c>
       <c r="C1785" t="s">
-        <v>273</v>
+        <v>361</v>
       </c>
       <c r="D1785" t="s">
-        <v>359</v>
+        <v>361</v>
       </c>
       <c r="E1785" t="s">
-        <v>13</v>
+        <v>361</v>
       </c>
       <c r="F1785" s="1">
         <v>0</v>
       </c>
       <c r="G1785" s="1">
-        <v>8601440</v>
+        <v>6.97229419303E9</v>
       </c>
       <c r="H1785" s="1">
-        <v>18873669</v>
+        <v>6.972294193030003E9</v>
       </c>
       <c r="I1785" s="1">
-        <v>-10272229</v>
-      </c>
-    </row>
-    <row r="1786" spans="1:9" ht="12.75">
-      <c r="A1786" t="s">
-        <v>312</v>
-      </c>
-      <c r="B1786" t="s">
-        <v>268</v>
-      </c>
-      <c r="C1786" t="s">
-        <v>296</v>
-      </c>
-      <c r="D1786" t="s">
-        <v>297</v>
-      </c>
-      <c r="E1786" t="s">
-        <v>13</v>
-      </c>
-      <c r="F1786" s="1">
-        <v>0</v>
-      </c>
-      <c r="G1786" s="1">
-        <v>2.2509215249E8</v>
-      </c>
-      <c r="H1786" s="1">
-        <v>2.2509215249E8</v>
-      </c>
-      <c r="I1786" s="1">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="1787" spans="1:9" ht="12.75">
-      <c r="A1787" t="s">
-        <v>312</v>
-      </c>
-      <c r="B1787" t="s">
-        <v>268</v>
-      </c>
-      <c r="C1787" t="s">
-        <v>296</v>
-      </c>
-      <c r="D1787" t="s">
-        <v>298</v>
-      </c>
-      <c r="E1787" t="s">
-        <v>13</v>
-      </c>
-      <c r="F1787" s="1">
-        <v>0</v>
-      </c>
-      <c r="G1787" s="1">
-        <v>0</v>
-      </c>
-      <c r="H1787" s="1">
-        <v>8826219.66</v>
-      </c>
-      <c r="I1787" s="1">
-        <v>-8826219.66</v>
-      </c>
-    </row>
-    <row r="1788" spans="1:9" ht="12.75">
-      <c r="A1788" t="s">
-        <v>360</v>
-      </c>
-      <c r="B1788" t="s">
-        <v>361</v>
-      </c>
-      <c r="C1788" t="s">
-        <v>361</v>
-      </c>
-      <c r="D1788" t="s">
-        <v>361</v>
-      </c>
-      <c r="E1788" t="s">
-        <v>361</v>
-      </c>
-      <c r="F1788" s="1">
-        <v>5.9604644775390625E-8</v>
-      </c>
-      <c r="G1788" s="1">
-        <v>6.97229419303E9</v>
-      </c>
-      <c r="H1788" s="1">
-        <v>6.972294193030003E9</v>
-      </c>
-      <c r="I1788" s="1">
-        <v>-2.5741755962371826E-6</v>
+        <v>-3.0510127544403076E-6</v>
       </c>
     </row>
   </sheetData>

</xml_diff>